<commit_message>
Add SHAP analysis for SVM
</commit_message>
<xml_diff>
--- a/outputs/xgb/rip_temperatura.xlsx
+++ b/outputs/xgb/rip_temperatura.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/u0186653/Desktop/research/dingen/deepnir/outputs/xgb/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43C102A4-818F-3248-9EF1-9706BDBEF000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C186DAD6-1741-F947-A31C-611BEF8C0644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38400" yWindow="-720" windowWidth="38400" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="mod unif" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="22">
   <si>
     <t>Crop</t>
   </si>
@@ -419,13 +420,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
@@ -437,41 +465,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -801,10 +802,10 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="22" t="s">
         <v>9</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -815,8 +816,8 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="15"/>
-      <c r="B3" s="18"/>
+      <c r="A3" s="24"/>
+      <c r="B3" s="19"/>
       <c r="C3" t="s">
         <v>18</v>
       </c>
@@ -825,8 +826,8 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="15"/>
-      <c r="B4" s="18"/>
+      <c r="A4" s="24"/>
+      <c r="B4" s="19"/>
       <c r="C4" t="s">
         <v>19</v>
       </c>
@@ -835,8 +836,8 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="15"/>
-      <c r="B5" s="19"/>
+      <c r="A5" s="24"/>
+      <c r="B5" s="20"/>
       <c r="C5" s="8" t="s">
         <v>20</v>
       </c>
@@ -845,8 +846,8 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="15"/>
-      <c r="B6" s="20" t="s">
+      <c r="A6" s="24"/>
+      <c r="B6" s="18" t="s">
         <v>10</v>
       </c>
       <c r="C6" s="7" t="s">
@@ -857,8 +858,8 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="15"/>
-      <c r="B7" s="18"/>
+      <c r="A7" s="24"/>
+      <c r="B7" s="19"/>
       <c r="C7" t="s">
         <v>18</v>
       </c>
@@ -867,8 +868,8 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="15"/>
-      <c r="B8" s="18"/>
+      <c r="A8" s="24"/>
+      <c r="B8" s="19"/>
       <c r="C8" t="s">
         <v>19</v>
       </c>
@@ -877,8 +878,8 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="15"/>
-      <c r="B9" s="19"/>
+      <c r="A9" s="24"/>
+      <c r="B9" s="20"/>
       <c r="C9" s="8" t="s">
         <v>20</v>
       </c>
@@ -887,8 +888,8 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="15"/>
-      <c r="B10" s="20" t="s">
+      <c r="A10" s="24"/>
+      <c r="B10" s="18" t="s">
         <v>11</v>
       </c>
       <c r="C10" s="7" t="s">
@@ -899,8 +900,8 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="15"/>
-      <c r="B11" s="18"/>
+      <c r="A11" s="24"/>
+      <c r="B11" s="19"/>
       <c r="C11" t="s">
         <v>18</v>
       </c>
@@ -909,8 +910,8 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="15"/>
-      <c r="B12" s="18"/>
+      <c r="A12" s="24"/>
+      <c r="B12" s="19"/>
       <c r="C12" t="s">
         <v>19</v>
       </c>
@@ -919,8 +920,8 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="15"/>
-      <c r="B13" s="19"/>
+      <c r="A13" s="24"/>
+      <c r="B13" s="20"/>
       <c r="C13" s="8" t="s">
         <v>20</v>
       </c>
@@ -929,8 +930,8 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="15"/>
-      <c r="B14" s="20" t="s">
+      <c r="A14" s="24"/>
+      <c r="B14" s="18" t="s">
         <v>12</v>
       </c>
       <c r="C14" s="7" t="s">
@@ -941,8 +942,8 @@
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="15"/>
-      <c r="B15" s="18"/>
+      <c r="A15" s="24"/>
+      <c r="B15" s="19"/>
       <c r="C15" t="s">
         <v>18</v>
       </c>
@@ -951,8 +952,8 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="15"/>
-      <c r="B16" s="18"/>
+      <c r="A16" s="24"/>
+      <c r="B16" s="19"/>
       <c r="C16" t="s">
         <v>19</v>
       </c>
@@ -961,8 +962,8 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="15"/>
-      <c r="B17" s="19"/>
+      <c r="A17" s="24"/>
+      <c r="B17" s="20"/>
       <c r="C17" s="8" t="s">
         <v>20</v>
       </c>
@@ -971,8 +972,8 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="15"/>
-      <c r="B18" s="20" t="s">
+      <c r="A18" s="24"/>
+      <c r="B18" s="18" t="s">
         <v>13</v>
       </c>
       <c r="C18" s="7" t="s">
@@ -983,8 +984,8 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="15"/>
-      <c r="B19" s="18"/>
+      <c r="A19" s="24"/>
+      <c r="B19" s="19"/>
       <c r="C19" t="s">
         <v>18</v>
       </c>
@@ -993,8 +994,8 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="15"/>
-      <c r="B20" s="18"/>
+      <c r="A20" s="24"/>
+      <c r="B20" s="19"/>
       <c r="C20" t="s">
         <v>19</v>
       </c>
@@ -1003,8 +1004,8 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="15"/>
-      <c r="B21" s="19"/>
+      <c r="A21" s="24"/>
+      <c r="B21" s="20"/>
       <c r="C21" s="8" t="s">
         <v>20</v>
       </c>
@@ -1013,8 +1014,8 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="15"/>
-      <c r="B22" s="20" t="s">
+      <c r="A22" s="24"/>
+      <c r="B22" s="18" t="s">
         <v>14</v>
       </c>
       <c r="C22" s="7" t="s">
@@ -1025,8 +1026,8 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="15"/>
-      <c r="B23" s="18"/>
+      <c r="A23" s="24"/>
+      <c r="B23" s="19"/>
       <c r="C23" t="s">
         <v>18</v>
       </c>
@@ -1035,8 +1036,8 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="15"/>
-      <c r="B24" s="18"/>
+      <c r="A24" s="24"/>
+      <c r="B24" s="19"/>
       <c r="C24" t="s">
         <v>19</v>
       </c>
@@ -1045,8 +1046,8 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="15"/>
-      <c r="B25" s="19"/>
+      <c r="A25" s="24"/>
+      <c r="B25" s="20"/>
       <c r="C25" s="8" t="s">
         <v>20</v>
       </c>
@@ -1055,8 +1056,8 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="15"/>
-      <c r="B26" s="20" t="s">
+      <c r="A26" s="24"/>
+      <c r="B26" s="18" t="s">
         <v>15</v>
       </c>
       <c r="C26" t="s">
@@ -1067,8 +1068,8 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="15"/>
-      <c r="B27" s="18"/>
+      <c r="A27" s="24"/>
+      <c r="B27" s="19"/>
       <c r="C27" t="s">
         <v>18</v>
       </c>
@@ -1077,8 +1078,8 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="15"/>
-      <c r="B28" s="18"/>
+      <c r="A28" s="24"/>
+      <c r="B28" s="19"/>
       <c r="C28" t="s">
         <v>19</v>
       </c>
@@ -1087,7 +1088,7 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="16"/>
+      <c r="A29" s="25"/>
       <c r="B29" s="21"/>
       <c r="C29" s="5" t="s">
         <v>20</v>
@@ -1097,10 +1098,10 @@
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="14" t="s">
+      <c r="A30" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="B30" s="17" t="s">
+      <c r="B30" s="22" t="s">
         <v>16</v>
       </c>
       <c r="C30" s="2" t="s">
@@ -1111,8 +1112,8 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="15"/>
-      <c r="B31" s="18"/>
+      <c r="A31" s="24"/>
+      <c r="B31" s="19"/>
       <c r="C31" t="s">
         <v>18</v>
       </c>
@@ -1121,8 +1122,8 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="15"/>
-      <c r="B32" s="18"/>
+      <c r="A32" s="24"/>
+      <c r="B32" s="19"/>
       <c r="C32" t="s">
         <v>19</v>
       </c>
@@ -1131,8 +1132,8 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="15"/>
-      <c r="B33" s="19"/>
+      <c r="A33" s="24"/>
+      <c r="B33" s="20"/>
       <c r="C33" s="8" t="s">
         <v>20</v>
       </c>
@@ -1141,8 +1142,8 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="15"/>
-      <c r="B34" s="20" t="s">
+      <c r="A34" s="24"/>
+      <c r="B34" s="18" t="s">
         <v>9</v>
       </c>
       <c r="C34" s="7" t="s">
@@ -1153,8 +1154,8 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="15"/>
-      <c r="B35" s="18"/>
+      <c r="A35" s="24"/>
+      <c r="B35" s="19"/>
       <c r="C35" t="s">
         <v>18</v>
       </c>
@@ -1163,8 +1164,8 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="15"/>
-      <c r="B36" s="18"/>
+      <c r="A36" s="24"/>
+      <c r="B36" s="19"/>
       <c r="C36" t="s">
         <v>19</v>
       </c>
@@ -1173,8 +1174,8 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="15"/>
-      <c r="B37" s="19"/>
+      <c r="A37" s="24"/>
+      <c r="B37" s="20"/>
       <c r="C37" s="8" t="s">
         <v>20</v>
       </c>
@@ -1183,8 +1184,8 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="15"/>
-      <c r="B38" s="20" t="s">
+      <c r="A38" s="24"/>
+      <c r="B38" s="18" t="s">
         <v>10</v>
       </c>
       <c r="C38" s="7" t="s">
@@ -1195,8 +1196,8 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="15"/>
-      <c r="B39" s="18"/>
+      <c r="A39" s="24"/>
+      <c r="B39" s="19"/>
       <c r="C39" t="s">
         <v>18</v>
       </c>
@@ -1205,8 +1206,8 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="15"/>
-      <c r="B40" s="18"/>
+      <c r="A40" s="24"/>
+      <c r="B40" s="19"/>
       <c r="C40" t="s">
         <v>19</v>
       </c>
@@ -1215,8 +1216,8 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="15"/>
-      <c r="B41" s="19"/>
+      <c r="A41" s="24"/>
+      <c r="B41" s="20"/>
       <c r="C41" s="8" t="s">
         <v>20</v>
       </c>
@@ -1225,8 +1226,8 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="15"/>
-      <c r="B42" s="20" t="s">
+      <c r="A42" s="24"/>
+      <c r="B42" s="18" t="s">
         <v>11</v>
       </c>
       <c r="C42" s="7" t="s">
@@ -1237,8 +1238,8 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" s="15"/>
-      <c r="B43" s="18"/>
+      <c r="A43" s="24"/>
+      <c r="B43" s="19"/>
       <c r="C43" t="s">
         <v>18</v>
       </c>
@@ -1247,8 +1248,8 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="15"/>
-      <c r="B44" s="18"/>
+      <c r="A44" s="24"/>
+      <c r="B44" s="19"/>
       <c r="C44" t="s">
         <v>19</v>
       </c>
@@ -1257,8 +1258,8 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="15"/>
-      <c r="B45" s="19"/>
+      <c r="A45" s="24"/>
+      <c r="B45" s="20"/>
       <c r="C45" s="8" t="s">
         <v>20</v>
       </c>
@@ -1267,8 +1268,8 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="15"/>
-      <c r="B46" s="20" t="s">
+      <c r="A46" s="24"/>
+      <c r="B46" s="18" t="s">
         <v>12</v>
       </c>
       <c r="C46" s="7" t="s">
@@ -1279,8 +1280,8 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="15"/>
-      <c r="B47" s="18"/>
+      <c r="A47" s="24"/>
+      <c r="B47" s="19"/>
       <c r="C47" t="s">
         <v>18</v>
       </c>
@@ -1289,8 +1290,8 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="15"/>
-      <c r="B48" s="18"/>
+      <c r="A48" s="24"/>
+      <c r="B48" s="19"/>
       <c r="C48" t="s">
         <v>19</v>
       </c>
@@ -1299,8 +1300,8 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="15"/>
-      <c r="B49" s="19"/>
+      <c r="A49" s="24"/>
+      <c r="B49" s="20"/>
       <c r="C49" s="8" t="s">
         <v>20</v>
       </c>
@@ -1309,8 +1310,8 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A50" s="15"/>
-      <c r="B50" s="20" t="s">
+      <c r="A50" s="24"/>
+      <c r="B50" s="18" t="s">
         <v>13</v>
       </c>
       <c r="C50" s="7" t="s">
@@ -1321,8 +1322,8 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A51" s="15"/>
-      <c r="B51" s="18"/>
+      <c r="A51" s="24"/>
+      <c r="B51" s="19"/>
       <c r="C51" t="s">
         <v>18</v>
       </c>
@@ -1331,8 +1332,8 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="15"/>
-      <c r="B52" s="18"/>
+      <c r="A52" s="24"/>
+      <c r="B52" s="19"/>
       <c r="C52" t="s">
         <v>19</v>
       </c>
@@ -1341,8 +1342,8 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="15"/>
-      <c r="B53" s="19"/>
+      <c r="A53" s="24"/>
+      <c r="B53" s="20"/>
       <c r="C53" s="8" t="s">
         <v>20</v>
       </c>
@@ -1351,8 +1352,8 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" s="15"/>
-      <c r="B54" s="20" t="s">
+      <c r="A54" s="24"/>
+      <c r="B54" s="18" t="s">
         <v>14</v>
       </c>
       <c r="C54" s="7" t="s">
@@ -1363,8 +1364,8 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" s="15"/>
-      <c r="B55" s="18"/>
+      <c r="A55" s="24"/>
+      <c r="B55" s="19"/>
       <c r="C55" t="s">
         <v>18</v>
       </c>
@@ -1373,8 +1374,8 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" s="15"/>
-      <c r="B56" s="18"/>
+      <c r="A56" s="24"/>
+      <c r="B56" s="19"/>
       <c r="C56" t="s">
         <v>19</v>
       </c>
@@ -1383,8 +1384,8 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" s="15"/>
-      <c r="B57" s="19"/>
+      <c r="A57" s="24"/>
+      <c r="B57" s="20"/>
       <c r="C57" s="8" t="s">
         <v>20</v>
       </c>
@@ -1393,8 +1394,8 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A58" s="15"/>
-      <c r="B58" s="20" t="s">
+      <c r="A58" s="24"/>
+      <c r="B58" s="18" t="s">
         <v>15</v>
       </c>
       <c r="C58" t="s">
@@ -1405,8 +1406,8 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A59" s="15"/>
-      <c r="B59" s="18"/>
+      <c r="A59" s="24"/>
+      <c r="B59" s="19"/>
       <c r="C59" t="s">
         <v>18</v>
       </c>
@@ -1415,8 +1416,8 @@
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" s="15"/>
-      <c r="B60" s="18"/>
+      <c r="A60" s="24"/>
+      <c r="B60" s="19"/>
       <c r="C60" t="s">
         <v>19</v>
       </c>
@@ -1425,7 +1426,7 @@
       </c>
     </row>
     <row r="61" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="16"/>
+      <c r="A61" s="25"/>
       <c r="B61" s="21"/>
       <c r="C61" s="5" t="s">
         <v>20</v>
@@ -1435,10 +1436,10 @@
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="11" t="s">
+      <c r="A62" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B62" s="22" t="s">
+      <c r="B62" s="17" t="s">
         <v>10</v>
       </c>
       <c r="C62" s="2" t="s">
@@ -1449,8 +1450,8 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="12"/>
-      <c r="B63" s="23"/>
+      <c r="A63" s="27"/>
+      <c r="B63" s="12"/>
       <c r="C63" t="s">
         <v>18</v>
       </c>
@@ -1459,8 +1460,8 @@
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="12"/>
-      <c r="B64" s="23"/>
+      <c r="A64" s="27"/>
+      <c r="B64" s="12"/>
       <c r="C64" t="s">
         <v>19</v>
       </c>
@@ -1469,8 +1470,8 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" s="12"/>
-      <c r="B65" s="24"/>
+      <c r="A65" s="27"/>
+      <c r="B65" s="13"/>
       <c r="C65" s="8" t="s">
         <v>20</v>
       </c>
@@ -1479,8 +1480,8 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" s="12"/>
-      <c r="B66" s="25" t="s">
+      <c r="A66" s="27"/>
+      <c r="B66" s="11" t="s">
         <v>12</v>
       </c>
       <c r="C66" s="7" t="s">
@@ -1491,8 +1492,8 @@
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" s="12"/>
-      <c r="B67" s="23"/>
+      <c r="A67" s="27"/>
+      <c r="B67" s="12"/>
       <c r="C67" t="s">
         <v>18</v>
       </c>
@@ -1501,8 +1502,8 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="12"/>
-      <c r="B68" s="23"/>
+      <c r="A68" s="27"/>
+      <c r="B68" s="12"/>
       <c r="C68" t="s">
         <v>19</v>
       </c>
@@ -1511,8 +1512,8 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" s="12"/>
-      <c r="B69" s="24"/>
+      <c r="A69" s="27"/>
+      <c r="B69" s="13"/>
       <c r="C69" s="8" t="s">
         <v>20</v>
       </c>
@@ -1521,8 +1522,8 @@
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="12"/>
-      <c r="B70" s="25" t="s">
+      <c r="A70" s="27"/>
+      <c r="B70" s="11" t="s">
         <v>14</v>
       </c>
       <c r="C70" t="s">
@@ -1533,8 +1534,8 @@
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" s="12"/>
-      <c r="B71" s="23"/>
+      <c r="A71" s="27"/>
+      <c r="B71" s="12"/>
       <c r="C71" t="s">
         <v>18</v>
       </c>
@@ -1543,8 +1544,8 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" s="12"/>
-      <c r="B72" s="23"/>
+      <c r="A72" s="27"/>
+      <c r="B72" s="12"/>
       <c r="C72" t="s">
         <v>19</v>
       </c>
@@ -1553,8 +1554,8 @@
       </c>
     </row>
     <row r="73" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="13"/>
-      <c r="B73" s="26"/>
+      <c r="A73" s="28"/>
+      <c r="B73" s="16"/>
       <c r="C73" s="5" t="s">
         <v>20</v>
       </c>
@@ -1563,10 +1564,10 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="11" t="s">
+      <c r="A74" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="B74" s="22" t="s">
+      <c r="B74" s="17" t="s">
         <v>16</v>
       </c>
       <c r="C74" s="2" t="s">
@@ -1577,8 +1578,8 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="12"/>
-      <c r="B75" s="23"/>
+      <c r="A75" s="27"/>
+      <c r="B75" s="12"/>
       <c r="C75" t="s">
         <v>18</v>
       </c>
@@ -1587,8 +1588,8 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="12"/>
-      <c r="B76" s="23"/>
+      <c r="A76" s="27"/>
+      <c r="B76" s="12"/>
       <c r="C76" t="s">
         <v>19</v>
       </c>
@@ -1597,8 +1598,8 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="12"/>
-      <c r="B77" s="24"/>
+      <c r="A77" s="27"/>
+      <c r="B77" s="13"/>
       <c r="C77" s="8" t="s">
         <v>20</v>
       </c>
@@ -1607,8 +1608,8 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="12"/>
-      <c r="B78" s="25" t="s">
+      <c r="A78" s="27"/>
+      <c r="B78" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C78" s="7" t="s">
@@ -1619,8 +1620,8 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="12"/>
-      <c r="B79" s="23"/>
+      <c r="A79" s="27"/>
+      <c r="B79" s="12"/>
       <c r="C79" t="s">
         <v>18</v>
       </c>
@@ -1629,8 +1630,8 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" s="12"/>
-      <c r="B80" s="23"/>
+      <c r="A80" s="27"/>
+      <c r="B80" s="12"/>
       <c r="C80" t="s">
         <v>19</v>
       </c>
@@ -1639,8 +1640,8 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A81" s="12"/>
-      <c r="B81" s="24"/>
+      <c r="A81" s="27"/>
+      <c r="B81" s="13"/>
       <c r="C81" s="8" t="s">
         <v>20</v>
       </c>
@@ -1649,8 +1650,8 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" s="12"/>
-      <c r="B82" s="25" t="s">
+      <c r="A82" s="27"/>
+      <c r="B82" s="11" t="s">
         <v>10</v>
       </c>
       <c r="C82" s="7" t="s">
@@ -1661,8 +1662,8 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" s="12"/>
-      <c r="B83" s="23"/>
+      <c r="A83" s="27"/>
+      <c r="B83" s="12"/>
       <c r="C83" t="s">
         <v>18</v>
       </c>
@@ -1671,8 +1672,8 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" s="12"/>
-      <c r="B84" s="23"/>
+      <c r="A84" s="27"/>
+      <c r="B84" s="12"/>
       <c r="C84" t="s">
         <v>19</v>
       </c>
@@ -1681,8 +1682,8 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A85" s="12"/>
-      <c r="B85" s="24"/>
+      <c r="A85" s="27"/>
+      <c r="B85" s="13"/>
       <c r="C85" s="8" t="s">
         <v>20</v>
       </c>
@@ -1691,8 +1692,8 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A86" s="12"/>
-      <c r="B86" s="25" t="s">
+      <c r="A86" s="27"/>
+      <c r="B86" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C86" s="7" t="s">
@@ -1703,8 +1704,8 @@
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A87" s="12"/>
-      <c r="B87" s="23"/>
+      <c r="A87" s="27"/>
+      <c r="B87" s="12"/>
       <c r="C87" t="s">
         <v>18</v>
       </c>
@@ -1713,8 +1714,8 @@
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A88" s="12"/>
-      <c r="B88" s="23"/>
+      <c r="A88" s="27"/>
+      <c r="B88" s="12"/>
       <c r="C88" t="s">
         <v>19</v>
       </c>
@@ -1723,8 +1724,8 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A89" s="12"/>
-      <c r="B89" s="24"/>
+      <c r="A89" s="27"/>
+      <c r="B89" s="13"/>
       <c r="C89" s="8" t="s">
         <v>20</v>
       </c>
@@ -1733,8 +1734,8 @@
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A90" s="12"/>
-      <c r="B90" s="25" t="s">
+      <c r="A90" s="27"/>
+      <c r="B90" s="11" t="s">
         <v>12</v>
       </c>
       <c r="C90" s="7" t="s">
@@ -1745,8 +1746,8 @@
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A91" s="12"/>
-      <c r="B91" s="23"/>
+      <c r="A91" s="27"/>
+      <c r="B91" s="12"/>
       <c r="C91" t="s">
         <v>18</v>
       </c>
@@ -1755,8 +1756,8 @@
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A92" s="12"/>
-      <c r="B92" s="23"/>
+      <c r="A92" s="27"/>
+      <c r="B92" s="12"/>
       <c r="C92" t="s">
         <v>19</v>
       </c>
@@ -1765,8 +1766,8 @@
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A93" s="12"/>
-      <c r="B93" s="24"/>
+      <c r="A93" s="27"/>
+      <c r="B93" s="13"/>
       <c r="C93" s="8" t="s">
         <v>20</v>
       </c>
@@ -1775,8 +1776,8 @@
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A94" s="12"/>
-      <c r="B94" s="25" t="s">
+      <c r="A94" s="27"/>
+      <c r="B94" s="11" t="s">
         <v>13</v>
       </c>
       <c r="C94" s="7" t="s">
@@ -1787,8 +1788,8 @@
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A95" s="12"/>
-      <c r="B95" s="23"/>
+      <c r="A95" s="27"/>
+      <c r="B95" s="12"/>
       <c r="C95" t="s">
         <v>18</v>
       </c>
@@ -1797,8 +1798,8 @@
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A96" s="12"/>
-      <c r="B96" s="23"/>
+      <c r="A96" s="27"/>
+      <c r="B96" s="12"/>
       <c r="C96" t="s">
         <v>19</v>
       </c>
@@ -1807,8 +1808,8 @@
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A97" s="12"/>
-      <c r="B97" s="24"/>
+      <c r="A97" s="27"/>
+      <c r="B97" s="13"/>
       <c r="C97" s="8" t="s">
         <v>20</v>
       </c>
@@ -1817,8 +1818,8 @@
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A98" s="12"/>
-      <c r="B98" s="25" t="s">
+      <c r="A98" s="27"/>
+      <c r="B98" s="11" t="s">
         <v>14</v>
       </c>
       <c r="C98" s="7" t="s">
@@ -1829,8 +1830,8 @@
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A99" s="12"/>
-      <c r="B99" s="23"/>
+      <c r="A99" s="27"/>
+      <c r="B99" s="12"/>
       <c r="C99" t="s">
         <v>18</v>
       </c>
@@ -1839,8 +1840,8 @@
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A100" s="12"/>
-      <c r="B100" s="23"/>
+      <c r="A100" s="27"/>
+      <c r="B100" s="12"/>
       <c r="C100" t="s">
         <v>19</v>
       </c>
@@ -1849,8 +1850,8 @@
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A101" s="12"/>
-      <c r="B101" s="24"/>
+      <c r="A101" s="27"/>
+      <c r="B101" s="13"/>
       <c r="C101" s="8" t="s">
         <v>20</v>
       </c>
@@ -1859,8 +1860,8 @@
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A102" s="12"/>
-      <c r="B102" s="25" t="s">
+      <c r="A102" s="27"/>
+      <c r="B102" s="11" t="s">
         <v>15</v>
       </c>
       <c r="C102" t="s">
@@ -1871,8 +1872,8 @@
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A103" s="12"/>
-      <c r="B103" s="23"/>
+      <c r="A103" s="27"/>
+      <c r="B103" s="12"/>
       <c r="C103" t="s">
         <v>18</v>
       </c>
@@ -1881,8 +1882,8 @@
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A104" s="12"/>
-      <c r="B104" s="23"/>
+      <c r="A104" s="27"/>
+      <c r="B104" s="12"/>
       <c r="C104" t="s">
         <v>19</v>
       </c>
@@ -1891,8 +1892,8 @@
       </c>
     </row>
     <row r="105" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="13"/>
-      <c r="B105" s="26"/>
+      <c r="A105" s="28"/>
+      <c r="B105" s="16"/>
       <c r="C105" s="5" t="s">
         <v>20</v>
       </c>
@@ -1901,10 +1902,10 @@
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A106" s="11" t="s">
+      <c r="A106" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="B106" s="22" t="s">
+      <c r="B106" s="17" t="s">
         <v>16</v>
       </c>
       <c r="C106" s="2" t="s">
@@ -1915,8 +1916,8 @@
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A107" s="12"/>
-      <c r="B107" s="23"/>
+      <c r="A107" s="27"/>
+      <c r="B107" s="12"/>
       <c r="C107" t="s">
         <v>18</v>
       </c>
@@ -1925,8 +1926,8 @@
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A108" s="12"/>
-      <c r="B108" s="23"/>
+      <c r="A108" s="27"/>
+      <c r="B108" s="12"/>
       <c r="C108" t="s">
         <v>19</v>
       </c>
@@ -1935,8 +1936,8 @@
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A109" s="12"/>
-      <c r="B109" s="24"/>
+      <c r="A109" s="27"/>
+      <c r="B109" s="13"/>
       <c r="C109" s="8" t="s">
         <v>20</v>
       </c>
@@ -1945,8 +1946,8 @@
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A110" s="12"/>
-      <c r="B110" s="25" t="s">
+      <c r="A110" s="27"/>
+      <c r="B110" s="11" t="s">
         <v>9</v>
       </c>
       <c r="C110" s="7" t="s">
@@ -1957,8 +1958,8 @@
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A111" s="12"/>
-      <c r="B111" s="23"/>
+      <c r="A111" s="27"/>
+      <c r="B111" s="12"/>
       <c r="C111" t="s">
         <v>18</v>
       </c>
@@ -1967,8 +1968,8 @@
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A112" s="12"/>
-      <c r="B112" s="23"/>
+      <c r="A112" s="27"/>
+      <c r="B112" s="12"/>
       <c r="C112" t="s">
         <v>19</v>
       </c>
@@ -1977,8 +1978,8 @@
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A113" s="12"/>
-      <c r="B113" s="24"/>
+      <c r="A113" s="27"/>
+      <c r="B113" s="13"/>
       <c r="C113" s="8" t="s">
         <v>20</v>
       </c>
@@ -1987,8 +1988,8 @@
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A114" s="12"/>
-      <c r="B114" s="25" t="s">
+      <c r="A114" s="27"/>
+      <c r="B114" s="11" t="s">
         <v>10</v>
       </c>
       <c r="C114" s="7" t="s">
@@ -1999,8 +2000,8 @@
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A115" s="12"/>
-      <c r="B115" s="23"/>
+      <c r="A115" s="27"/>
+      <c r="B115" s="12"/>
       <c r="C115" t="s">
         <v>18</v>
       </c>
@@ -2009,8 +2010,8 @@
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A116" s="12"/>
-      <c r="B116" s="23"/>
+      <c r="A116" s="27"/>
+      <c r="B116" s="12"/>
       <c r="C116" t="s">
         <v>19</v>
       </c>
@@ -2019,8 +2020,8 @@
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A117" s="12"/>
-      <c r="B117" s="24"/>
+      <c r="A117" s="27"/>
+      <c r="B117" s="13"/>
       <c r="C117" s="8" t="s">
         <v>20</v>
       </c>
@@ -2029,8 +2030,8 @@
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A118" s="12"/>
-      <c r="B118" s="25" t="s">
+      <c r="A118" s="27"/>
+      <c r="B118" s="11" t="s">
         <v>11</v>
       </c>
       <c r="C118" s="7" t="s">
@@ -2041,8 +2042,8 @@
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A119" s="12"/>
-      <c r="B119" s="23"/>
+      <c r="A119" s="27"/>
+      <c r="B119" s="12"/>
       <c r="C119" t="s">
         <v>18</v>
       </c>
@@ -2051,8 +2052,8 @@
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A120" s="12"/>
-      <c r="B120" s="23"/>
+      <c r="A120" s="27"/>
+      <c r="B120" s="12"/>
       <c r="C120" t="s">
         <v>19</v>
       </c>
@@ -2061,8 +2062,8 @@
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A121" s="12"/>
-      <c r="B121" s="24"/>
+      <c r="A121" s="27"/>
+      <c r="B121" s="13"/>
       <c r="C121" s="8" t="s">
         <v>20</v>
       </c>
@@ -2071,8 +2072,8 @@
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A122" s="12"/>
-      <c r="B122" s="25" t="s">
+      <c r="A122" s="27"/>
+      <c r="B122" s="11" t="s">
         <v>12</v>
       </c>
       <c r="C122" s="7" t="s">
@@ -2083,8 +2084,8 @@
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A123" s="12"/>
-      <c r="B123" s="23"/>
+      <c r="A123" s="27"/>
+      <c r="B123" s="12"/>
       <c r="C123" t="s">
         <v>18</v>
       </c>
@@ -2093,8 +2094,8 @@
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A124" s="12"/>
-      <c r="B124" s="23"/>
+      <c r="A124" s="27"/>
+      <c r="B124" s="12"/>
       <c r="C124" t="s">
         <v>19</v>
       </c>
@@ -2103,8 +2104,8 @@
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A125" s="12"/>
-      <c r="B125" s="24"/>
+      <c r="A125" s="27"/>
+      <c r="B125" s="13"/>
       <c r="C125" s="8" t="s">
         <v>20</v>
       </c>
@@ -2113,8 +2114,8 @@
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A126" s="12"/>
-      <c r="B126" s="25" t="s">
+      <c r="A126" s="27"/>
+      <c r="B126" s="11" t="s">
         <v>13</v>
       </c>
       <c r="C126" s="7" t="s">
@@ -2125,8 +2126,8 @@
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A127" s="12"/>
-      <c r="B127" s="23"/>
+      <c r="A127" s="27"/>
+      <c r="B127" s="12"/>
       <c r="C127" t="s">
         <v>18</v>
       </c>
@@ -2135,8 +2136,8 @@
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A128" s="12"/>
-      <c r="B128" s="23"/>
+      <c r="A128" s="27"/>
+      <c r="B128" s="12"/>
       <c r="C128" t="s">
         <v>19</v>
       </c>
@@ -2145,8 +2146,8 @@
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A129" s="12"/>
-      <c r="B129" s="24"/>
+      <c r="A129" s="27"/>
+      <c r="B129" s="13"/>
       <c r="C129" s="8" t="s">
         <v>20</v>
       </c>
@@ -2155,8 +2156,8 @@
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A130" s="12"/>
-      <c r="B130" s="25" t="s">
+      <c r="A130" s="27"/>
+      <c r="B130" s="11" t="s">
         <v>14</v>
       </c>
       <c r="C130" t="s">
@@ -2167,8 +2168,8 @@
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A131" s="12"/>
-      <c r="B131" s="27"/>
+      <c r="A131" s="27"/>
+      <c r="B131" s="14"/>
       <c r="C131" t="s">
         <v>18</v>
       </c>
@@ -2177,8 +2178,8 @@
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A132" s="12"/>
-      <c r="B132" s="27"/>
+      <c r="A132" s="27"/>
+      <c r="B132" s="14"/>
       <c r="C132" t="s">
         <v>19</v>
       </c>
@@ -2187,8 +2188,8 @@
       </c>
     </row>
     <row r="133" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A133" s="13"/>
-      <c r="B133" s="28"/>
+      <c r="A133" s="28"/>
+      <c r="B133" s="15"/>
       <c r="C133" s="5" t="s">
         <v>20</v>
       </c>
@@ -2198,6 +2199,34 @@
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="A106:A133"/>
+    <mergeCell ref="B2:B5"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="B42:B45"/>
+    <mergeCell ref="A2:A29"/>
+    <mergeCell ref="A30:A61"/>
+    <mergeCell ref="A62:A73"/>
+    <mergeCell ref="A74:A105"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="B90:B93"/>
+    <mergeCell ref="B46:B49"/>
+    <mergeCell ref="B50:B53"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="B58:B61"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="B66:B69"/>
+    <mergeCell ref="B70:B73"/>
+    <mergeCell ref="B74:B77"/>
+    <mergeCell ref="B78:B81"/>
+    <mergeCell ref="B82:B85"/>
+    <mergeCell ref="B86:B89"/>
     <mergeCell ref="B118:B121"/>
     <mergeCell ref="B122:B125"/>
     <mergeCell ref="B126:B129"/>
@@ -2208,34 +2237,1482 @@
     <mergeCell ref="B106:B109"/>
     <mergeCell ref="B110:B113"/>
     <mergeCell ref="B114:B117"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D2:D133">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="num" val="0.3"/>
+        <color theme="6" tint="0.39997558519241921"/>
+        <color theme="9" tint="0.39997558519241921"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33A4ED39-B87F-1743-8E8A-8F63746863B4}">
+  <dimension ref="A1:D133"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.1640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="23" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="3">
+        <v>0.1301015674738594</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="24"/>
+      <c r="B3" s="19"/>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" s="4">
+        <v>0.13402608829122681</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="24"/>
+      <c r="B4" s="19"/>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="4">
+        <v>0.13494775766629541</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="24"/>
+      <c r="B5" s="20"/>
+      <c r="C5" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" s="9">
+        <v>0.13588219107194779</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="24"/>
+      <c r="B6" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="10">
+        <v>8.7197393343593527E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="24"/>
+      <c r="B7" s="19"/>
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="4">
+        <v>8.9251540503721721E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="24"/>
+      <c r="B8" s="19"/>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="4">
+        <v>9.3732085132325615E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="24"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="9">
+        <v>9.1071714917428895E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="24"/>
+      <c r="B10" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="10">
+        <v>6.8627642004529407E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="24"/>
+      <c r="B11" s="19"/>
+      <c r="C11" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="4">
+        <v>7.0697798536253978E-2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="24"/>
+      <c r="B12" s="19"/>
+      <c r="C12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="4">
+        <v>7.1183972508996135E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="24"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="9">
+        <v>7.1676879416155928E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="24"/>
+      <c r="B14" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D14" s="10">
+        <v>2.413884789904178</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="24"/>
+      <c r="B15" s="19"/>
+      <c r="C15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="4">
+        <v>2.4802627520053711</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="24"/>
+      <c r="B16" s="19"/>
+      <c r="C16" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" s="4">
+        <v>2.49658010750582</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="24"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D17" s="9">
+        <v>2.511439073037633</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" s="24"/>
+      <c r="B18" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D18" s="10">
+        <v>0.20216304294312201</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" s="24"/>
+      <c r="B19" s="19"/>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="4">
+        <v>0.211137631567758</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" s="24"/>
+      <c r="B20" s="19"/>
+      <c r="C20" t="s">
+        <v>19</v>
+      </c>
+      <c r="D20" s="4">
+        <v>0.20430665986244179</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" s="24"/>
+      <c r="B21" s="20"/>
+      <c r="C21" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" s="9">
+        <v>0.2140616380060881</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="24"/>
+      <c r="B22" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D22" s="10">
+        <v>0.2054388351861943</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" s="24"/>
+      <c r="B23" s="19"/>
+      <c r="C23" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="4">
+        <v>0.2116359087575479</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" s="24"/>
+      <c r="B24" s="19"/>
+      <c r="C24" t="s">
+        <v>19</v>
+      </c>
+      <c r="D24" s="4">
+        <v>0.2155780518977212</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" s="24"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" s="9">
+        <v>0.21029613778829159</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" s="24"/>
+      <c r="B26" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" t="s">
+        <v>17</v>
+      </c>
+      <c r="D26" s="4">
+        <v>0.25376462146063528</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" s="24"/>
+      <c r="B27" s="19"/>
+      <c r="C27" t="s">
+        <v>18</v>
+      </c>
+      <c r="D27" s="4">
+        <v>0.2615280021098641</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" s="24"/>
+      <c r="B28" s="19"/>
+      <c r="C28" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="4">
+        <v>0.26990480614255008</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="25"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D29" s="6">
+        <v>0.27167776452277481</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" s="23" t="s">
+        <v>5</v>
+      </c>
+      <c r="B30" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D30" s="3">
+        <v>3.6100573187706451E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" s="24"/>
+      <c r="B31" s="19"/>
+      <c r="C31" t="s">
+        <v>18</v>
+      </c>
+      <c r="D31" s="4">
+        <v>4.2207636335963868E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" s="24"/>
+      <c r="B32" s="19"/>
+      <c r="C32" t="s">
+        <v>19</v>
+      </c>
+      <c r="D32" s="4">
+        <v>3.4067810029911813E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" s="24"/>
+      <c r="B33" s="20"/>
+      <c r="C33" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="9">
+        <v>4.1325069029110872E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" s="24"/>
+      <c r="B34" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D34" s="10">
+        <v>9.455865750465706E-3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" s="24"/>
+      <c r="B35" s="19"/>
+      <c r="C35" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35" s="4">
+        <v>9.5126151323139639E-3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" s="24"/>
+      <c r="B36" s="19"/>
+      <c r="C36" t="s">
+        <v>19</v>
+      </c>
+      <c r="D36" s="4">
+        <v>9.534072158928205E-3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" s="24"/>
+      <c r="B37" s="20"/>
+      <c r="C37" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D37" s="9">
+        <v>9.5269090694023381E-3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" s="24"/>
+      <c r="B38" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D38" s="10">
+        <v>3.7380655162108638E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" s="24"/>
+      <c r="B39" s="19"/>
+      <c r="C39" t="s">
+        <v>18</v>
+      </c>
+      <c r="D39" s="4">
+        <v>3.7604995178085299E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" s="24"/>
+      <c r="B40" s="19"/>
+      <c r="C40" t="s">
+        <v>19</v>
+      </c>
+      <c r="D40" s="4">
+        <v>3.7689818475479482E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" s="24"/>
+      <c r="B41" s="20"/>
+      <c r="C41" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D41" s="9">
+        <v>3.7661501557015538E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" s="24"/>
+      <c r="B42" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D42" s="10">
+        <v>6.5096077147390644E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" s="24"/>
+      <c r="B43" s="19"/>
+      <c r="C43" t="s">
+        <v>18</v>
+      </c>
+      <c r="D43" s="4">
+        <v>6.6755789165110491E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" s="24"/>
+      <c r="B44" s="19"/>
+      <c r="C44" t="s">
+        <v>19</v>
+      </c>
+      <c r="D44" s="4">
+        <v>6.5634465755376598E-2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" s="24"/>
+      <c r="B45" s="20"/>
+      <c r="C45" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D45" s="9">
+        <v>6.68560983900017E-2</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" s="24"/>
+      <c r="B46" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D46" s="10">
+        <v>0.61233770838430968</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" s="24"/>
+      <c r="B47" s="19"/>
+      <c r="C47" t="s">
+        <v>18</v>
+      </c>
+      <c r="D47" s="4">
+        <v>0.62535794623704755</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" s="24"/>
+      <c r="B48" s="19"/>
+      <c r="C48" t="s">
+        <v>19</v>
+      </c>
+      <c r="D48" s="4">
+        <v>0.62426402156514327</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" s="24"/>
+      <c r="B49" s="20"/>
+      <c r="C49" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D49" s="9">
+        <v>0.6278080298970462</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" s="24"/>
+      <c r="B50" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D50" s="10">
+        <v>0.1152057775715053</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" s="24"/>
+      <c r="B51" s="19"/>
+      <c r="C51" t="s">
+        <v>18</v>
+      </c>
+      <c r="D51" s="4">
+        <v>0.1152720383388694</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" s="24"/>
+      <c r="B52" s="19"/>
+      <c r="C52" t="s">
+        <v>19</v>
+      </c>
+      <c r="D52" s="4">
+        <v>0.1145828935436736</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" s="24"/>
+      <c r="B53" s="20"/>
+      <c r="C53" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D53" s="9">
+        <v>0.11363205024839609</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" s="24"/>
+      <c r="B54" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D54" s="10">
+        <v>0.2735418850232379</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" s="24"/>
+      <c r="B55" s="19"/>
+      <c r="C55" t="s">
+        <v>18</v>
+      </c>
+      <c r="D55" s="4">
+        <v>0.27920965493753808</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" s="24"/>
+      <c r="B56" s="19"/>
+      <c r="C56" t="s">
+        <v>19</v>
+      </c>
+      <c r="D56" s="4">
+        <v>0.27488113345956439</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" s="24"/>
+      <c r="B57" s="20"/>
+      <c r="C57" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D57" s="9">
+        <v>0.2790743385733383</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" s="24"/>
+      <c r="B58" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="C58" t="s">
+        <v>17</v>
+      </c>
+      <c r="D58" s="4">
+        <v>0.26461766959125638</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" s="24"/>
+      <c r="B59" s="19"/>
+      <c r="C59" t="s">
+        <v>18</v>
+      </c>
+      <c r="D59" s="4">
+        <v>0.27245008578804858</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" s="24"/>
+      <c r="B60" s="19"/>
+      <c r="C60" t="s">
+        <v>19</v>
+      </c>
+      <c r="D60" s="4">
+        <v>0.27844823392710288</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="25"/>
+      <c r="B61" s="21"/>
+      <c r="C61" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D61" s="6">
+        <v>0.2658439882709781</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" s="26" t="s">
+        <v>6</v>
+      </c>
+      <c r="B62" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D62" s="3">
+        <v>8.2996792888149415E-2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" s="27"/>
+      <c r="B63" s="12"/>
+      <c r="C63" t="s">
+        <v>18</v>
+      </c>
+      <c r="D63" s="4">
+        <v>7.6630334846993026E-2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" s="27"/>
+      <c r="B64" s="12"/>
+      <c r="C64" t="s">
+        <v>19</v>
+      </c>
+      <c r="D64" s="4">
+        <v>8.7566188313433019E-2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" s="27"/>
+      <c r="B65" s="13"/>
+      <c r="C65" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D65" s="9">
+        <v>9.0736291612686482E-2</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" s="27"/>
+      <c r="B66" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D66" s="10">
+        <v>0.17265201756948931</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A67" s="27"/>
+      <c r="B67" s="12"/>
+      <c r="C67" t="s">
+        <v>18</v>
+      </c>
+      <c r="D67" s="4">
+        <v>0.1752346954688084</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" s="27"/>
+      <c r="B68" s="12"/>
+      <c r="C68" t="s">
+        <v>19</v>
+      </c>
+      <c r="D68" s="4">
+        <v>0.1770890308705948</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A69" s="27"/>
+      <c r="B69" s="13"/>
+      <c r="C69" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D69" s="9">
+        <v>0.1851935758003197</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A70" s="27"/>
+      <c r="B70" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C70" t="s">
+        <v>21</v>
+      </c>
+      <c r="D70" s="4">
+        <v>0.71497307863846904</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A71" s="27"/>
+      <c r="B71" s="12"/>
+      <c r="C71" t="s">
+        <v>18</v>
+      </c>
+      <c r="D71" s="4">
+        <v>0.72566826306088428</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A72" s="27"/>
+      <c r="B72" s="12"/>
+      <c r="C72" t="s">
+        <v>19</v>
+      </c>
+      <c r="D72" s="4">
+        <v>0.73334729229962403</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A73" s="28"/>
+      <c r="B73" s="16"/>
+      <c r="C73" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D73" s="6">
+        <v>0.75181593778566647</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A74" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="B74" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D74" s="3">
+        <v>0.24385458884060629</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" s="27"/>
+      <c r="B75" s="12"/>
+      <c r="C75" t="s">
+        <v>18</v>
+      </c>
+      <c r="D75" s="4">
+        <v>0.24894748113851631</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A76" s="27"/>
+      <c r="B76" s="12"/>
+      <c r="C76" t="s">
+        <v>19</v>
+      </c>
+      <c r="D76" s="4">
+        <v>0.25000946826032999</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" s="27"/>
+      <c r="B77" s="13"/>
+      <c r="C77" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D77" s="9">
+        <v>0.25370729950083282</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A78" s="27"/>
+      <c r="B78" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C78" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D78" s="10">
+        <v>7.5389045948129091E-2</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" s="27"/>
+      <c r="B79" s="12"/>
+      <c r="C79" t="s">
+        <v>18</v>
+      </c>
+      <c r="D79" s="4">
+        <v>7.7725739605658886E-2</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A80" s="27"/>
+      <c r="B80" s="12"/>
+      <c r="C80" t="s">
+        <v>19</v>
+      </c>
+      <c r="D80" s="4">
+        <v>7.7291862251832294E-2</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A81" s="27"/>
+      <c r="B81" s="13"/>
+      <c r="C81" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D81" s="9">
+        <v>7.8435068006639352E-2</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A82" s="27"/>
+      <c r="B82" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C82" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D82" s="10">
+        <v>1.1412545149931459E-2</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A83" s="27"/>
+      <c r="B83" s="12"/>
+      <c r="C83" t="s">
+        <v>18</v>
+      </c>
+      <c r="D83" s="4">
+        <v>1.1650895650407909E-2</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A84" s="27"/>
+      <c r="B84" s="12"/>
+      <c r="C84" t="s">
+        <v>19</v>
+      </c>
+      <c r="D84" s="4">
+        <v>1.170059730266702E-2</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A85" s="27"/>
+      <c r="B85" s="13"/>
+      <c r="C85" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D85" s="9">
+        <v>1.187365808528223E-2</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A86" s="27"/>
+      <c r="B86" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C86" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D86" s="10">
+        <v>5.7078267598780437E-2</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A87" s="27"/>
+      <c r="B87" s="12"/>
+      <c r="C87" t="s">
+        <v>18</v>
+      </c>
+      <c r="D87" s="4">
+        <v>5.9350140326845963E-2</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A88" s="27"/>
+      <c r="B88" s="12"/>
+      <c r="C88" t="s">
+        <v>19</v>
+      </c>
+      <c r="D88" s="4">
+        <v>6.2130406959769638E-2</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A89" s="27"/>
+      <c r="B89" s="13"/>
+      <c r="C89" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D89" s="9">
+        <v>6.3049363195466099E-2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A90" s="27"/>
+      <c r="B90" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C90" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D90" s="10">
+        <v>0.22927071284321909</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A91" s="27"/>
+      <c r="B91" s="12"/>
+      <c r="C91" t="s">
+        <v>18</v>
+      </c>
+      <c r="D91" s="4">
+        <v>0.23550334018943589</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A92" s="27"/>
+      <c r="B92" s="12"/>
+      <c r="C92" t="s">
+        <v>19</v>
+      </c>
+      <c r="D92" s="4">
+        <v>0.23593244881465511</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A93" s="27"/>
+      <c r="B93" s="13"/>
+      <c r="C93" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D93" s="9">
+        <v>0.2394220701715819</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A94" s="27"/>
+      <c r="B94" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C94" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D94" s="10">
+        <v>9.5105931762187387E-2</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A95" s="27"/>
+      <c r="B95" s="12"/>
+      <c r="C95" t="s">
+        <v>18</v>
+      </c>
+      <c r="D95" s="4">
+        <v>9.7647607853982313E-2</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A96" s="27"/>
+      <c r="B96" s="12"/>
+      <c r="C96" t="s">
+        <v>19</v>
+      </c>
+      <c r="D96" s="4">
+        <v>9.7770162040637196E-2</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A97" s="27"/>
+      <c r="B97" s="13"/>
+      <c r="C97" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D97" s="9">
+        <v>9.9216257510935241E-2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A98" s="27"/>
+      <c r="B98" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C98" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D98" s="10">
+        <v>0.24743543087857439</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A99" s="27"/>
+      <c r="B99" s="12"/>
+      <c r="C99" t="s">
+        <v>18</v>
+      </c>
+      <c r="D99" s="4">
+        <v>0.25542011092194411</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A100" s="27"/>
+      <c r="B100" s="12"/>
+      <c r="C100" t="s">
+        <v>19</v>
+      </c>
+      <c r="D100" s="4">
+        <v>0.253680690598581</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A101" s="27"/>
+      <c r="B101" s="13"/>
+      <c r="C101" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D101" s="9">
+        <v>0.25556104695814158</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A102" s="27"/>
+      <c r="B102" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C102" t="s">
+        <v>21</v>
+      </c>
+      <c r="D102" s="4">
+        <v>0.47723873313025528</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A103" s="27"/>
+      <c r="B103" s="12"/>
+      <c r="C103" t="s">
+        <v>18</v>
+      </c>
+      <c r="D103" s="4">
+        <v>0.44138329429964063</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A104" s="27"/>
+      <c r="B104" s="12"/>
+      <c r="C104" t="s">
+        <v>19</v>
+      </c>
+      <c r="D104" s="4">
+        <v>0.48672689308359057</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="28"/>
+      <c r="B105" s="16"/>
+      <c r="C105" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D105" s="6">
+        <v>0.43333226984197443</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A106" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="B106" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D106" s="3">
+        <v>1.2297599007838139E-2</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A107" s="27"/>
+      <c r="B107" s="12"/>
+      <c r="C107" t="s">
+        <v>18</v>
+      </c>
+      <c r="D107" s="4">
+        <v>1.270535662377249E-2</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A108" s="27"/>
+      <c r="B108" s="12"/>
+      <c r="C108" t="s">
+        <v>19</v>
+      </c>
+      <c r="D108" s="4">
+        <v>1.2865324868177101E-2</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A109" s="27"/>
+      <c r="B109" s="13"/>
+      <c r="C109" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D109" s="9">
+        <v>1.2934413686034591E-2</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A110" s="27"/>
+      <c r="B110" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C110" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D110" s="10">
+        <v>9.1574332907111186E-2</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A111" s="27"/>
+      <c r="B111" s="12"/>
+      <c r="C111" t="s">
+        <v>18</v>
+      </c>
+      <c r="D111" s="4">
+        <v>9.8268736010668586E-2</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A112" s="27"/>
+      <c r="B112" s="12"/>
+      <c r="C112" t="s">
+        <v>19</v>
+      </c>
+      <c r="D112" s="4">
+        <v>9.5801915616672575E-2</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A113" s="27"/>
+      <c r="B113" s="13"/>
+      <c r="C113" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D113" s="9">
+        <v>9.8397679652662884E-2</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A114" s="27"/>
+      <c r="B114" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C114" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D114" s="10">
+        <v>0.45828203664566808</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A115" s="27"/>
+      <c r="B115" s="12"/>
+      <c r="C115" t="s">
+        <v>18</v>
+      </c>
+      <c r="D115" s="4">
+        <v>0.43165024367147758</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A116" s="27"/>
+      <c r="B116" s="12"/>
+      <c r="C116" t="s">
+        <v>19</v>
+      </c>
+      <c r="D116" s="4">
+        <v>0.45029990593925873</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A117" s="27"/>
+      <c r="B117" s="13"/>
+      <c r="C117" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D117" s="9">
+        <v>0.45271808725231938</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A118" s="27"/>
+      <c r="B118" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C118" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D118" s="10">
+        <v>0.4595088402256316</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A119" s="27"/>
+      <c r="B119" s="12"/>
+      <c r="C119" t="s">
+        <v>18</v>
+      </c>
+      <c r="D119" s="4">
+        <v>0.46748205873421811</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A120" s="27"/>
+      <c r="B120" s="12"/>
+      <c r="C120" t="s">
+        <v>19</v>
+      </c>
+      <c r="D120" s="4">
+        <v>0.47196243064906568</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A121" s="27"/>
+      <c r="B121" s="13"/>
+      <c r="C121" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D121" s="9">
+        <v>0.47449694312665941</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A122" s="27"/>
+      <c r="B122" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C122" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D122" s="10">
+        <v>0.80397012545017332</v>
+      </c>
+    </row>
+    <row r="123" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A123" s="27"/>
+      <c r="B123" s="12"/>
+      <c r="C123" t="s">
+        <v>18</v>
+      </c>
+      <c r="D123" s="4">
+        <v>0.86941118966212549</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A124" s="27"/>
+      <c r="B124" s="12"/>
+      <c r="C124" t="s">
+        <v>19</v>
+      </c>
+      <c r="D124" s="4">
+        <v>0.86499810537187616</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A125" s="27"/>
+      <c r="B125" s="13"/>
+      <c r="C125" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D125" s="9">
+        <v>0.85986466255963501</v>
+      </c>
+    </row>
+    <row r="126" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A126" s="27"/>
+      <c r="B126" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C126" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="D126" s="10">
+        <v>3.4305146799567502E-3</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A127" s="27"/>
+      <c r="B127" s="12"/>
+      <c r="C127" t="s">
+        <v>18</v>
+      </c>
+      <c r="D127" s="4">
+        <v>3.5442619639945009E-3</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A128" s="27"/>
+      <c r="B128" s="12"/>
+      <c r="C128" t="s">
+        <v>19</v>
+      </c>
+      <c r="D128" s="4">
+        <v>3.588886399252731E-3</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A129" s="27"/>
+      <c r="B129" s="13"/>
+      <c r="C129" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D129" s="9">
+        <v>3.6081592836369031E-3</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A130" s="27"/>
+      <c r="B130" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C130" t="s">
+        <v>21</v>
+      </c>
+      <c r="D130" s="4">
+        <v>0.77816652260410979</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A131" s="27"/>
+      <c r="B131" s="14"/>
+      <c r="C131" t="s">
+        <v>18</v>
+      </c>
+      <c r="D131" s="4">
+        <v>0.78419970675528083</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A132" s="27"/>
+      <c r="B132" s="14"/>
+      <c r="C132" t="s">
+        <v>19</v>
+      </c>
+      <c r="D132" s="4">
+        <v>0.79407326277318413</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A133" s="28"/>
+      <c r="B133" s="15"/>
+      <c r="C133" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D133" s="6">
+        <v>0.79833756107729781</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="38">
+    <mergeCell ref="B130:B133"/>
+    <mergeCell ref="B94:B97"/>
+    <mergeCell ref="B98:B101"/>
+    <mergeCell ref="B102:B105"/>
+    <mergeCell ref="A106:A133"/>
+    <mergeCell ref="B106:B109"/>
+    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="B114:B117"/>
+    <mergeCell ref="B118:B121"/>
+    <mergeCell ref="B122:B125"/>
+    <mergeCell ref="B126:B129"/>
+    <mergeCell ref="A62:A73"/>
+    <mergeCell ref="B62:B65"/>
+    <mergeCell ref="B66:B69"/>
     <mergeCell ref="B70:B73"/>
+    <mergeCell ref="A74:A105"/>
     <mergeCell ref="B74:B77"/>
     <mergeCell ref="B78:B81"/>
     <mergeCell ref="B82:B85"/>
     <mergeCell ref="B86:B89"/>
     <mergeCell ref="B90:B93"/>
+    <mergeCell ref="A30:A61"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="B42:B45"/>
     <mergeCell ref="B46:B49"/>
     <mergeCell ref="B50:B53"/>
     <mergeCell ref="B54:B57"/>
     <mergeCell ref="B58:B61"/>
-    <mergeCell ref="B62:B65"/>
-    <mergeCell ref="B66:B69"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="B42:B45"/>
     <mergeCell ref="A2:A29"/>
-    <mergeCell ref="A30:A61"/>
-    <mergeCell ref="A62:A73"/>
-    <mergeCell ref="A74:A105"/>
-    <mergeCell ref="A106:A133"/>
     <mergeCell ref="B2:B5"/>
     <mergeCell ref="B6:B9"/>
     <mergeCell ref="B10:B13"/>
     <mergeCell ref="B14:B17"/>
     <mergeCell ref="B18:B21"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="B26:B29"/>
   </mergeCells>
   <conditionalFormatting sqref="D2:D133">
     <cfRule type="colorScale" priority="1">

</xml_diff>

<commit_message>
Add temperature repeatability for SVM
</commit_message>
<xml_diff>
--- a/outputs/xgb/rip_temperatura.xlsx
+++ b/outputs/xgb/rip_temperatura.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/u0186653/Desktop/research/dingen/deepnir/outputs/xgb/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C186DAD6-1741-F947-A31C-611BEF8C0644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2BAFEFA-D8D3-4143-9AB8-D4375E7960A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="mod unif" sheetId="2" r:id="rId2"/>
+    <sheet name="modelli singoli" sheetId="1" r:id="rId1"/>
+    <sheet name="modello unificato" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -453,6 +453,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -465,20 +474,42 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -802,10 +833,10 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="25" t="s">
         <v>9</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -816,7 +847,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="24"/>
+      <c r="A3" s="27"/>
       <c r="B3" s="19"/>
       <c r="C3" t="s">
         <v>18</v>
@@ -826,7 +857,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="24"/>
+      <c r="A4" s="27"/>
       <c r="B4" s="19"/>
       <c r="C4" t="s">
         <v>19</v>
@@ -836,7 +867,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="24"/>
+      <c r="A5" s="27"/>
       <c r="B5" s="20"/>
       <c r="C5" s="8" t="s">
         <v>20</v>
@@ -846,7 +877,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="24"/>
+      <c r="A6" s="27"/>
       <c r="B6" s="18" t="s">
         <v>10</v>
       </c>
@@ -858,7 +889,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="24"/>
+      <c r="A7" s="27"/>
       <c r="B7" s="19"/>
       <c r="C7" t="s">
         <v>18</v>
@@ -868,7 +899,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="24"/>
+      <c r="A8" s="27"/>
       <c r="B8" s="19"/>
       <c r="C8" t="s">
         <v>19</v>
@@ -878,7 +909,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="24"/>
+      <c r="A9" s="27"/>
       <c r="B9" s="20"/>
       <c r="C9" s="8" t="s">
         <v>20</v>
@@ -888,7 +919,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="24"/>
+      <c r="A10" s="27"/>
       <c r="B10" s="18" t="s">
         <v>11</v>
       </c>
@@ -900,7 +931,7 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="24"/>
+      <c r="A11" s="27"/>
       <c r="B11" s="19"/>
       <c r="C11" t="s">
         <v>18</v>
@@ -910,7 +941,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="24"/>
+      <c r="A12" s="27"/>
       <c r="B12" s="19"/>
       <c r="C12" t="s">
         <v>19</v>
@@ -920,7 +951,7 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="24"/>
+      <c r="A13" s="27"/>
       <c r="B13" s="20"/>
       <c r="C13" s="8" t="s">
         <v>20</v>
@@ -930,7 +961,7 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="24"/>
+      <c r="A14" s="27"/>
       <c r="B14" s="18" t="s">
         <v>12</v>
       </c>
@@ -942,7 +973,7 @@
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="24"/>
+      <c r="A15" s="27"/>
       <c r="B15" s="19"/>
       <c r="C15" t="s">
         <v>18</v>
@@ -952,7 +983,7 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="24"/>
+      <c r="A16" s="27"/>
       <c r="B16" s="19"/>
       <c r="C16" t="s">
         <v>19</v>
@@ -962,7 +993,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="24"/>
+      <c r="A17" s="27"/>
       <c r="B17" s="20"/>
       <c r="C17" s="8" t="s">
         <v>20</v>
@@ -972,7 +1003,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="24"/>
+      <c r="A18" s="27"/>
       <c r="B18" s="18" t="s">
         <v>13</v>
       </c>
@@ -984,7 +1015,7 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="24"/>
+      <c r="A19" s="27"/>
       <c r="B19" s="19"/>
       <c r="C19" t="s">
         <v>18</v>
@@ -994,7 +1025,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="24"/>
+      <c r="A20" s="27"/>
       <c r="B20" s="19"/>
       <c r="C20" t="s">
         <v>19</v>
@@ -1004,7 +1035,7 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="24"/>
+      <c r="A21" s="27"/>
       <c r="B21" s="20"/>
       <c r="C21" s="8" t="s">
         <v>20</v>
@@ -1014,7 +1045,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="24"/>
+      <c r="A22" s="27"/>
       <c r="B22" s="18" t="s">
         <v>14</v>
       </c>
@@ -1026,7 +1057,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="24"/>
+      <c r="A23" s="27"/>
       <c r="B23" s="19"/>
       <c r="C23" t="s">
         <v>18</v>
@@ -1036,7 +1067,7 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="24"/>
+      <c r="A24" s="27"/>
       <c r="B24" s="19"/>
       <c r="C24" t="s">
         <v>19</v>
@@ -1046,7 +1077,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="24"/>
+      <c r="A25" s="27"/>
       <c r="B25" s="20"/>
       <c r="C25" s="8" t="s">
         <v>20</v>
@@ -1056,7 +1087,7 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="24"/>
+      <c r="A26" s="27"/>
       <c r="B26" s="18" t="s">
         <v>15</v>
       </c>
@@ -1068,7 +1099,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="24"/>
+      <c r="A27" s="27"/>
       <c r="B27" s="19"/>
       <c r="C27" t="s">
         <v>18</v>
@@ -1078,7 +1109,7 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="24"/>
+      <c r="A28" s="27"/>
       <c r="B28" s="19"/>
       <c r="C28" t="s">
         <v>19</v>
@@ -1088,7 +1119,7 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="25"/>
+      <c r="A29" s="28"/>
       <c r="B29" s="21"/>
       <c r="C29" s="5" t="s">
         <v>20</v>
@@ -1098,10 +1129,10 @@
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="23" t="s">
+      <c r="A30" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="B30" s="22" t="s">
+      <c r="B30" s="25" t="s">
         <v>16</v>
       </c>
       <c r="C30" s="2" t="s">
@@ -1112,7 +1143,7 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="24"/>
+      <c r="A31" s="27"/>
       <c r="B31" s="19"/>
       <c r="C31" t="s">
         <v>18</v>
@@ -1122,7 +1153,7 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="24"/>
+      <c r="A32" s="27"/>
       <c r="B32" s="19"/>
       <c r="C32" t="s">
         <v>19</v>
@@ -1132,7 +1163,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="24"/>
+      <c r="A33" s="27"/>
       <c r="B33" s="20"/>
       <c r="C33" s="8" t="s">
         <v>20</v>
@@ -1142,7 +1173,7 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="24"/>
+      <c r="A34" s="27"/>
       <c r="B34" s="18" t="s">
         <v>9</v>
       </c>
@@ -1154,7 +1185,7 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="24"/>
+      <c r="A35" s="27"/>
       <c r="B35" s="19"/>
       <c r="C35" t="s">
         <v>18</v>
@@ -1164,7 +1195,7 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="24"/>
+      <c r="A36" s="27"/>
       <c r="B36" s="19"/>
       <c r="C36" t="s">
         <v>19</v>
@@ -1174,7 +1205,7 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="24"/>
+      <c r="A37" s="27"/>
       <c r="B37" s="20"/>
       <c r="C37" s="8" t="s">
         <v>20</v>
@@ -1184,7 +1215,7 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="24"/>
+      <c r="A38" s="27"/>
       <c r="B38" s="18" t="s">
         <v>10</v>
       </c>
@@ -1196,7 +1227,7 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="24"/>
+      <c r="A39" s="27"/>
       <c r="B39" s="19"/>
       <c r="C39" t="s">
         <v>18</v>
@@ -1206,7 +1237,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="24"/>
+      <c r="A40" s="27"/>
       <c r="B40" s="19"/>
       <c r="C40" t="s">
         <v>19</v>
@@ -1216,7 +1247,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="24"/>
+      <c r="A41" s="27"/>
       <c r="B41" s="20"/>
       <c r="C41" s="8" t="s">
         <v>20</v>
@@ -1226,7 +1257,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="24"/>
+      <c r="A42" s="27"/>
       <c r="B42" s="18" t="s">
         <v>11</v>
       </c>
@@ -1238,7 +1269,7 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" s="24"/>
+      <c r="A43" s="27"/>
       <c r="B43" s="19"/>
       <c r="C43" t="s">
         <v>18</v>
@@ -1248,7 +1279,7 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="24"/>
+      <c r="A44" s="27"/>
       <c r="B44" s="19"/>
       <c r="C44" t="s">
         <v>19</v>
@@ -1258,7 +1289,7 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="24"/>
+      <c r="A45" s="27"/>
       <c r="B45" s="20"/>
       <c r="C45" s="8" t="s">
         <v>20</v>
@@ -1268,7 +1299,7 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="24"/>
+      <c r="A46" s="27"/>
       <c r="B46" s="18" t="s">
         <v>12</v>
       </c>
@@ -1280,7 +1311,7 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="24"/>
+      <c r="A47" s="27"/>
       <c r="B47" s="19"/>
       <c r="C47" t="s">
         <v>18</v>
@@ -1290,7 +1321,7 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="24"/>
+      <c r="A48" s="27"/>
       <c r="B48" s="19"/>
       <c r="C48" t="s">
         <v>19</v>
@@ -1300,7 +1331,7 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="24"/>
+      <c r="A49" s="27"/>
       <c r="B49" s="20"/>
       <c r="C49" s="8" t="s">
         <v>20</v>
@@ -1310,7 +1341,7 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A50" s="24"/>
+      <c r="A50" s="27"/>
       <c r="B50" s="18" t="s">
         <v>13</v>
       </c>
@@ -1322,7 +1353,7 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A51" s="24"/>
+      <c r="A51" s="27"/>
       <c r="B51" s="19"/>
       <c r="C51" t="s">
         <v>18</v>
@@ -1332,7 +1363,7 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="24"/>
+      <c r="A52" s="27"/>
       <c r="B52" s="19"/>
       <c r="C52" t="s">
         <v>19</v>
@@ -1342,7 +1373,7 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="24"/>
+      <c r="A53" s="27"/>
       <c r="B53" s="20"/>
       <c r="C53" s="8" t="s">
         <v>20</v>
@@ -1352,7 +1383,7 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" s="24"/>
+      <c r="A54" s="27"/>
       <c r="B54" s="18" t="s">
         <v>14</v>
       </c>
@@ -1364,7 +1395,7 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" s="24"/>
+      <c r="A55" s="27"/>
       <c r="B55" s="19"/>
       <c r="C55" t="s">
         <v>18</v>
@@ -1374,7 +1405,7 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" s="24"/>
+      <c r="A56" s="27"/>
       <c r="B56" s="19"/>
       <c r="C56" t="s">
         <v>19</v>
@@ -1384,7 +1415,7 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" s="24"/>
+      <c r="A57" s="27"/>
       <c r="B57" s="20"/>
       <c r="C57" s="8" t="s">
         <v>20</v>
@@ -1394,7 +1425,7 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A58" s="24"/>
+      <c r="A58" s="27"/>
       <c r="B58" s="18" t="s">
         <v>15</v>
       </c>
@@ -1406,7 +1437,7 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A59" s="24"/>
+      <c r="A59" s="27"/>
       <c r="B59" s="19"/>
       <c r="C59" t="s">
         <v>18</v>
@@ -1416,7 +1447,7 @@
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" s="24"/>
+      <c r="A60" s="27"/>
       <c r="B60" s="19"/>
       <c r="C60" t="s">
         <v>19</v>
@@ -1426,7 +1457,7 @@
       </c>
     </row>
     <row r="61" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="25"/>
+      <c r="A61" s="28"/>
       <c r="B61" s="21"/>
       <c r="C61" s="5" t="s">
         <v>20</v>
@@ -1436,7 +1467,7 @@
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="26" t="s">
+      <c r="A62" s="22" t="s">
         <v>6</v>
       </c>
       <c r="B62" s="17" t="s">
@@ -1450,7 +1481,7 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="27"/>
+      <c r="A63" s="23"/>
       <c r="B63" s="12"/>
       <c r="C63" t="s">
         <v>18</v>
@@ -1460,7 +1491,7 @@
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="27"/>
+      <c r="A64" s="23"/>
       <c r="B64" s="12"/>
       <c r="C64" t="s">
         <v>19</v>
@@ -1470,7 +1501,7 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" s="27"/>
+      <c r="A65" s="23"/>
       <c r="B65" s="13"/>
       <c r="C65" s="8" t="s">
         <v>20</v>
@@ -1480,7 +1511,7 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" s="27"/>
+      <c r="A66" s="23"/>
       <c r="B66" s="11" t="s">
         <v>12</v>
       </c>
@@ -1492,7 +1523,7 @@
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" s="27"/>
+      <c r="A67" s="23"/>
       <c r="B67" s="12"/>
       <c r="C67" t="s">
         <v>18</v>
@@ -1502,7 +1533,7 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="27"/>
+      <c r="A68" s="23"/>
       <c r="B68" s="12"/>
       <c r="C68" t="s">
         <v>19</v>
@@ -1512,7 +1543,7 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" s="27"/>
+      <c r="A69" s="23"/>
       <c r="B69" s="13"/>
       <c r="C69" s="8" t="s">
         <v>20</v>
@@ -1522,7 +1553,7 @@
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="27"/>
+      <c r="A70" s="23"/>
       <c r="B70" s="11" t="s">
         <v>14</v>
       </c>
@@ -1534,7 +1565,7 @@
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" s="27"/>
+      <c r="A71" s="23"/>
       <c r="B71" s="12"/>
       <c r="C71" t="s">
         <v>18</v>
@@ -1544,7 +1575,7 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" s="27"/>
+      <c r="A72" s="23"/>
       <c r="B72" s="12"/>
       <c r="C72" t="s">
         <v>19</v>
@@ -1554,7 +1585,7 @@
       </c>
     </row>
     <row r="73" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="28"/>
+      <c r="A73" s="24"/>
       <c r="B73" s="16"/>
       <c r="C73" s="5" t="s">
         <v>20</v>
@@ -1564,7 +1595,7 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="26" t="s">
+      <c r="A74" s="22" t="s">
         <v>7</v>
       </c>
       <c r="B74" s="17" t="s">
@@ -1578,7 +1609,7 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="27"/>
+      <c r="A75" s="23"/>
       <c r="B75" s="12"/>
       <c r="C75" t="s">
         <v>18</v>
@@ -1588,7 +1619,7 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="27"/>
+      <c r="A76" s="23"/>
       <c r="B76" s="12"/>
       <c r="C76" t="s">
         <v>19</v>
@@ -1598,7 +1629,7 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="27"/>
+      <c r="A77" s="23"/>
       <c r="B77" s="13"/>
       <c r="C77" s="8" t="s">
         <v>20</v>
@@ -1608,7 +1639,7 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="27"/>
+      <c r="A78" s="23"/>
       <c r="B78" s="11" t="s">
         <v>9</v>
       </c>
@@ -1620,7 +1651,7 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="27"/>
+      <c r="A79" s="23"/>
       <c r="B79" s="12"/>
       <c r="C79" t="s">
         <v>18</v>
@@ -1630,7 +1661,7 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" s="27"/>
+      <c r="A80" s="23"/>
       <c r="B80" s="12"/>
       <c r="C80" t="s">
         <v>19</v>
@@ -1640,7 +1671,7 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A81" s="27"/>
+      <c r="A81" s="23"/>
       <c r="B81" s="13"/>
       <c r="C81" s="8" t="s">
         <v>20</v>
@@ -1650,7 +1681,7 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" s="27"/>
+      <c r="A82" s="23"/>
       <c r="B82" s="11" t="s">
         <v>10</v>
       </c>
@@ -1662,7 +1693,7 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" s="27"/>
+      <c r="A83" s="23"/>
       <c r="B83" s="12"/>
       <c r="C83" t="s">
         <v>18</v>
@@ -1672,7 +1703,7 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" s="27"/>
+      <c r="A84" s="23"/>
       <c r="B84" s="12"/>
       <c r="C84" t="s">
         <v>19</v>
@@ -1682,7 +1713,7 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A85" s="27"/>
+      <c r="A85" s="23"/>
       <c r="B85" s="13"/>
       <c r="C85" s="8" t="s">
         <v>20</v>
@@ -1692,7 +1723,7 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A86" s="27"/>
+      <c r="A86" s="23"/>
       <c r="B86" s="11" t="s">
         <v>11</v>
       </c>
@@ -1704,7 +1735,7 @@
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A87" s="27"/>
+      <c r="A87" s="23"/>
       <c r="B87" s="12"/>
       <c r="C87" t="s">
         <v>18</v>
@@ -1714,7 +1745,7 @@
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A88" s="27"/>
+      <c r="A88" s="23"/>
       <c r="B88" s="12"/>
       <c r="C88" t="s">
         <v>19</v>
@@ -1724,7 +1755,7 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A89" s="27"/>
+      <c r="A89" s="23"/>
       <c r="B89" s="13"/>
       <c r="C89" s="8" t="s">
         <v>20</v>
@@ -1734,7 +1765,7 @@
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A90" s="27"/>
+      <c r="A90" s="23"/>
       <c r="B90" s="11" t="s">
         <v>12</v>
       </c>
@@ -1746,7 +1777,7 @@
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A91" s="27"/>
+      <c r="A91" s="23"/>
       <c r="B91" s="12"/>
       <c r="C91" t="s">
         <v>18</v>
@@ -1756,7 +1787,7 @@
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A92" s="27"/>
+      <c r="A92" s="23"/>
       <c r="B92" s="12"/>
       <c r="C92" t="s">
         <v>19</v>
@@ -1766,7 +1797,7 @@
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A93" s="27"/>
+      <c r="A93" s="23"/>
       <c r="B93" s="13"/>
       <c r="C93" s="8" t="s">
         <v>20</v>
@@ -1776,7 +1807,7 @@
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A94" s="27"/>
+      <c r="A94" s="23"/>
       <c r="B94" s="11" t="s">
         <v>13</v>
       </c>
@@ -1788,7 +1819,7 @@
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A95" s="27"/>
+      <c r="A95" s="23"/>
       <c r="B95" s="12"/>
       <c r="C95" t="s">
         <v>18</v>
@@ -1798,7 +1829,7 @@
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A96" s="27"/>
+      <c r="A96" s="23"/>
       <c r="B96" s="12"/>
       <c r="C96" t="s">
         <v>19</v>
@@ -1808,7 +1839,7 @@
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A97" s="27"/>
+      <c r="A97" s="23"/>
       <c r="B97" s="13"/>
       <c r="C97" s="8" t="s">
         <v>20</v>
@@ -1818,7 +1849,7 @@
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A98" s="27"/>
+      <c r="A98" s="23"/>
       <c r="B98" s="11" t="s">
         <v>14</v>
       </c>
@@ -1830,7 +1861,7 @@
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A99" s="27"/>
+      <c r="A99" s="23"/>
       <c r="B99" s="12"/>
       <c r="C99" t="s">
         <v>18</v>
@@ -1840,7 +1871,7 @@
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A100" s="27"/>
+      <c r="A100" s="23"/>
       <c r="B100" s="12"/>
       <c r="C100" t="s">
         <v>19</v>
@@ -1850,7 +1881,7 @@
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A101" s="27"/>
+      <c r="A101" s="23"/>
       <c r="B101" s="13"/>
       <c r="C101" s="8" t="s">
         <v>20</v>
@@ -1860,7 +1891,7 @@
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A102" s="27"/>
+      <c r="A102" s="23"/>
       <c r="B102" s="11" t="s">
         <v>15</v>
       </c>
@@ -1872,7 +1903,7 @@
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A103" s="27"/>
+      <c r="A103" s="23"/>
       <c r="B103" s="12"/>
       <c r="C103" t="s">
         <v>18</v>
@@ -1882,7 +1913,7 @@
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A104" s="27"/>
+      <c r="A104" s="23"/>
       <c r="B104" s="12"/>
       <c r="C104" t="s">
         <v>19</v>
@@ -1892,7 +1923,7 @@
       </c>
     </row>
     <row r="105" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="28"/>
+      <c r="A105" s="24"/>
       <c r="B105" s="16"/>
       <c r="C105" s="5" t="s">
         <v>20</v>
@@ -1902,7 +1933,7 @@
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A106" s="26" t="s">
+      <c r="A106" s="22" t="s">
         <v>8</v>
       </c>
       <c r="B106" s="17" t="s">
@@ -1916,7 +1947,7 @@
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A107" s="27"/>
+      <c r="A107" s="23"/>
       <c r="B107" s="12"/>
       <c r="C107" t="s">
         <v>18</v>
@@ -1926,7 +1957,7 @@
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A108" s="27"/>
+      <c r="A108" s="23"/>
       <c r="B108" s="12"/>
       <c r="C108" t="s">
         <v>19</v>
@@ -1936,7 +1967,7 @@
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A109" s="27"/>
+      <c r="A109" s="23"/>
       <c r="B109" s="13"/>
       <c r="C109" s="8" t="s">
         <v>20</v>
@@ -1946,7 +1977,7 @@
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A110" s="27"/>
+      <c r="A110" s="23"/>
       <c r="B110" s="11" t="s">
         <v>9</v>
       </c>
@@ -1958,7 +1989,7 @@
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A111" s="27"/>
+      <c r="A111" s="23"/>
       <c r="B111" s="12"/>
       <c r="C111" t="s">
         <v>18</v>
@@ -1968,7 +1999,7 @@
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A112" s="27"/>
+      <c r="A112" s="23"/>
       <c r="B112" s="12"/>
       <c r="C112" t="s">
         <v>19</v>
@@ -1978,7 +2009,7 @@
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A113" s="27"/>
+      <c r="A113" s="23"/>
       <c r="B113" s="13"/>
       <c r="C113" s="8" t="s">
         <v>20</v>
@@ -1988,7 +2019,7 @@
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A114" s="27"/>
+      <c r="A114" s="23"/>
       <c r="B114" s="11" t="s">
         <v>10</v>
       </c>
@@ -2000,7 +2031,7 @@
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A115" s="27"/>
+      <c r="A115" s="23"/>
       <c r="B115" s="12"/>
       <c r="C115" t="s">
         <v>18</v>
@@ -2010,7 +2041,7 @@
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A116" s="27"/>
+      <c r="A116" s="23"/>
       <c r="B116" s="12"/>
       <c r="C116" t="s">
         <v>19</v>
@@ -2020,7 +2051,7 @@
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A117" s="27"/>
+      <c r="A117" s="23"/>
       <c r="B117" s="13"/>
       <c r="C117" s="8" t="s">
         <v>20</v>
@@ -2030,7 +2061,7 @@
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A118" s="27"/>
+      <c r="A118" s="23"/>
       <c r="B118" s="11" t="s">
         <v>11</v>
       </c>
@@ -2042,7 +2073,7 @@
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A119" s="27"/>
+      <c r="A119" s="23"/>
       <c r="B119" s="12"/>
       <c r="C119" t="s">
         <v>18</v>
@@ -2052,7 +2083,7 @@
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A120" s="27"/>
+      <c r="A120" s="23"/>
       <c r="B120" s="12"/>
       <c r="C120" t="s">
         <v>19</v>
@@ -2062,7 +2093,7 @@
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A121" s="27"/>
+      <c r="A121" s="23"/>
       <c r="B121" s="13"/>
       <c r="C121" s="8" t="s">
         <v>20</v>
@@ -2072,7 +2103,7 @@
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A122" s="27"/>
+      <c r="A122" s="23"/>
       <c r="B122" s="11" t="s">
         <v>12</v>
       </c>
@@ -2084,7 +2115,7 @@
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A123" s="27"/>
+      <c r="A123" s="23"/>
       <c r="B123" s="12"/>
       <c r="C123" t="s">
         <v>18</v>
@@ -2094,7 +2125,7 @@
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A124" s="27"/>
+      <c r="A124" s="23"/>
       <c r="B124" s="12"/>
       <c r="C124" t="s">
         <v>19</v>
@@ -2104,7 +2135,7 @@
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A125" s="27"/>
+      <c r="A125" s="23"/>
       <c r="B125" s="13"/>
       <c r="C125" s="8" t="s">
         <v>20</v>
@@ -2114,7 +2145,7 @@
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A126" s="27"/>
+      <c r="A126" s="23"/>
       <c r="B126" s="11" t="s">
         <v>13</v>
       </c>
@@ -2126,7 +2157,7 @@
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A127" s="27"/>
+      <c r="A127" s="23"/>
       <c r="B127" s="12"/>
       <c r="C127" t="s">
         <v>18</v>
@@ -2136,7 +2167,7 @@
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A128" s="27"/>
+      <c r="A128" s="23"/>
       <c r="B128" s="12"/>
       <c r="C128" t="s">
         <v>19</v>
@@ -2146,7 +2177,7 @@
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A129" s="27"/>
+      <c r="A129" s="23"/>
       <c r="B129" s="13"/>
       <c r="C129" s="8" t="s">
         <v>20</v>
@@ -2156,7 +2187,7 @@
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A130" s="27"/>
+      <c r="A130" s="23"/>
       <c r="B130" s="11" t="s">
         <v>14</v>
       </c>
@@ -2168,7 +2199,7 @@
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A131" s="27"/>
+      <c r="A131" s="23"/>
       <c r="B131" s="14"/>
       <c r="C131" t="s">
         <v>18</v>
@@ -2178,7 +2209,7 @@
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A132" s="27"/>
+      <c r="A132" s="23"/>
       <c r="B132" s="14"/>
       <c r="C132" t="s">
         <v>19</v>
@@ -2188,7 +2219,7 @@
       </c>
     </row>
     <row r="133" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A133" s="28"/>
+      <c r="A133" s="24"/>
       <c r="B133" s="15"/>
       <c r="C133" s="5" t="s">
         <v>20</v>
@@ -2239,13 +2270,13 @@
     <mergeCell ref="B114:B117"/>
   </mergeCells>
   <conditionalFormatting sqref="D2:D133">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0.3"/>
-        <color theme="6" tint="0.39997558519241921"/>
-        <color theme="9" tint="0.39997558519241921"/>
-      </colorScale>
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="greaterThan">
+      <formula>0.3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:E133">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
+      <formula>1</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2278,10 +2309,10 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="25" t="s">
         <v>9</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -2292,7 +2323,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="24"/>
+      <c r="A3" s="27"/>
       <c r="B3" s="19"/>
       <c r="C3" t="s">
         <v>18</v>
@@ -2302,7 +2333,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="24"/>
+      <c r="A4" s="27"/>
       <c r="B4" s="19"/>
       <c r="C4" t="s">
         <v>19</v>
@@ -2312,7 +2343,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="24"/>
+      <c r="A5" s="27"/>
       <c r="B5" s="20"/>
       <c r="C5" s="8" t="s">
         <v>20</v>
@@ -2322,7 +2353,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="24"/>
+      <c r="A6" s="27"/>
       <c r="B6" s="18" t="s">
         <v>10</v>
       </c>
@@ -2334,7 +2365,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="24"/>
+      <c r="A7" s="27"/>
       <c r="B7" s="19"/>
       <c r="C7" t="s">
         <v>18</v>
@@ -2344,7 +2375,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="24"/>
+      <c r="A8" s="27"/>
       <c r="B8" s="19"/>
       <c r="C8" t="s">
         <v>19</v>
@@ -2354,7 +2385,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="24"/>
+      <c r="A9" s="27"/>
       <c r="B9" s="20"/>
       <c r="C9" s="8" t="s">
         <v>20</v>
@@ -2364,7 +2395,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="24"/>
+      <c r="A10" s="27"/>
       <c r="B10" s="18" t="s">
         <v>11</v>
       </c>
@@ -2376,7 +2407,7 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="24"/>
+      <c r="A11" s="27"/>
       <c r="B11" s="19"/>
       <c r="C11" t="s">
         <v>18</v>
@@ -2386,7 +2417,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="24"/>
+      <c r="A12" s="27"/>
       <c r="B12" s="19"/>
       <c r="C12" t="s">
         <v>19</v>
@@ -2396,7 +2427,7 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="24"/>
+      <c r="A13" s="27"/>
       <c r="B13" s="20"/>
       <c r="C13" s="8" t="s">
         <v>20</v>
@@ -2406,7 +2437,7 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="24"/>
+      <c r="A14" s="27"/>
       <c r="B14" s="18" t="s">
         <v>12</v>
       </c>
@@ -2418,7 +2449,7 @@
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="24"/>
+      <c r="A15" s="27"/>
       <c r="B15" s="19"/>
       <c r="C15" t="s">
         <v>18</v>
@@ -2428,7 +2459,7 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="24"/>
+      <c r="A16" s="27"/>
       <c r="B16" s="19"/>
       <c r="C16" t="s">
         <v>19</v>
@@ -2438,7 +2469,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="24"/>
+      <c r="A17" s="27"/>
       <c r="B17" s="20"/>
       <c r="C17" s="8" t="s">
         <v>20</v>
@@ -2448,7 +2479,7 @@
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="24"/>
+      <c r="A18" s="27"/>
       <c r="B18" s="18" t="s">
         <v>13</v>
       </c>
@@ -2460,7 +2491,7 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="24"/>
+      <c r="A19" s="27"/>
       <c r="B19" s="19"/>
       <c r="C19" t="s">
         <v>18</v>
@@ -2470,7 +2501,7 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="24"/>
+      <c r="A20" s="27"/>
       <c r="B20" s="19"/>
       <c r="C20" t="s">
         <v>19</v>
@@ -2480,7 +2511,7 @@
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="24"/>
+      <c r="A21" s="27"/>
       <c r="B21" s="20"/>
       <c r="C21" s="8" t="s">
         <v>20</v>
@@ -2490,7 +2521,7 @@
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="24"/>
+      <c r="A22" s="27"/>
       <c r="B22" s="18" t="s">
         <v>14</v>
       </c>
@@ -2502,7 +2533,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="24"/>
+      <c r="A23" s="27"/>
       <c r="B23" s="19"/>
       <c r="C23" t="s">
         <v>18</v>
@@ -2512,7 +2543,7 @@
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="24"/>
+      <c r="A24" s="27"/>
       <c r="B24" s="19"/>
       <c r="C24" t="s">
         <v>19</v>
@@ -2522,7 +2553,7 @@
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="24"/>
+      <c r="A25" s="27"/>
       <c r="B25" s="20"/>
       <c r="C25" s="8" t="s">
         <v>20</v>
@@ -2532,7 +2563,7 @@
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="24"/>
+      <c r="A26" s="27"/>
       <c r="B26" s="18" t="s">
         <v>15</v>
       </c>
@@ -2544,7 +2575,7 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="24"/>
+      <c r="A27" s="27"/>
       <c r="B27" s="19"/>
       <c r="C27" t="s">
         <v>18</v>
@@ -2554,7 +2585,7 @@
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="24"/>
+      <c r="A28" s="27"/>
       <c r="B28" s="19"/>
       <c r="C28" t="s">
         <v>19</v>
@@ -2564,7 +2595,7 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="25"/>
+      <c r="A29" s="28"/>
       <c r="B29" s="21"/>
       <c r="C29" s="5" t="s">
         <v>20</v>
@@ -2574,10 +2605,10 @@
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="23" t="s">
+      <c r="A30" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="B30" s="22" t="s">
+      <c r="B30" s="25" t="s">
         <v>16</v>
       </c>
       <c r="C30" s="2" t="s">
@@ -2588,7 +2619,7 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="24"/>
+      <c r="A31" s="27"/>
       <c r="B31" s="19"/>
       <c r="C31" t="s">
         <v>18</v>
@@ -2598,7 +2629,7 @@
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="24"/>
+      <c r="A32" s="27"/>
       <c r="B32" s="19"/>
       <c r="C32" t="s">
         <v>19</v>
@@ -2608,7 +2639,7 @@
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="24"/>
+      <c r="A33" s="27"/>
       <c r="B33" s="20"/>
       <c r="C33" s="8" t="s">
         <v>20</v>
@@ -2618,7 +2649,7 @@
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="24"/>
+      <c r="A34" s="27"/>
       <c r="B34" s="18" t="s">
         <v>9</v>
       </c>
@@ -2630,7 +2661,7 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="24"/>
+      <c r="A35" s="27"/>
       <c r="B35" s="19"/>
       <c r="C35" t="s">
         <v>18</v>
@@ -2640,7 +2671,7 @@
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="24"/>
+      <c r="A36" s="27"/>
       <c r="B36" s="19"/>
       <c r="C36" t="s">
         <v>19</v>
@@ -2650,7 +2681,7 @@
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="24"/>
+      <c r="A37" s="27"/>
       <c r="B37" s="20"/>
       <c r="C37" s="8" t="s">
         <v>20</v>
@@ -2660,7 +2691,7 @@
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="24"/>
+      <c r="A38" s="27"/>
       <c r="B38" s="18" t="s">
         <v>10</v>
       </c>
@@ -2672,7 +2703,7 @@
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="24"/>
+      <c r="A39" s="27"/>
       <c r="B39" s="19"/>
       <c r="C39" t="s">
         <v>18</v>
@@ -2682,7 +2713,7 @@
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="24"/>
+      <c r="A40" s="27"/>
       <c r="B40" s="19"/>
       <c r="C40" t="s">
         <v>19</v>
@@ -2692,7 +2723,7 @@
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="24"/>
+      <c r="A41" s="27"/>
       <c r="B41" s="20"/>
       <c r="C41" s="8" t="s">
         <v>20</v>
@@ -2702,7 +2733,7 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="24"/>
+      <c r="A42" s="27"/>
       <c r="B42" s="18" t="s">
         <v>11</v>
       </c>
@@ -2714,7 +2745,7 @@
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" s="24"/>
+      <c r="A43" s="27"/>
       <c r="B43" s="19"/>
       <c r="C43" t="s">
         <v>18</v>
@@ -2724,7 +2755,7 @@
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="24"/>
+      <c r="A44" s="27"/>
       <c r="B44" s="19"/>
       <c r="C44" t="s">
         <v>19</v>
@@ -2734,7 +2765,7 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="24"/>
+      <c r="A45" s="27"/>
       <c r="B45" s="20"/>
       <c r="C45" s="8" t="s">
         <v>20</v>
@@ -2744,7 +2775,7 @@
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="24"/>
+      <c r="A46" s="27"/>
       <c r="B46" s="18" t="s">
         <v>12</v>
       </c>
@@ -2756,7 +2787,7 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="24"/>
+      <c r="A47" s="27"/>
       <c r="B47" s="19"/>
       <c r="C47" t="s">
         <v>18</v>
@@ -2766,7 +2797,7 @@
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="24"/>
+      <c r="A48" s="27"/>
       <c r="B48" s="19"/>
       <c r="C48" t="s">
         <v>19</v>
@@ -2776,7 +2807,7 @@
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="24"/>
+      <c r="A49" s="27"/>
       <c r="B49" s="20"/>
       <c r="C49" s="8" t="s">
         <v>20</v>
@@ -2786,7 +2817,7 @@
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A50" s="24"/>
+      <c r="A50" s="27"/>
       <c r="B50" s="18" t="s">
         <v>13</v>
       </c>
@@ -2798,7 +2829,7 @@
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A51" s="24"/>
+      <c r="A51" s="27"/>
       <c r="B51" s="19"/>
       <c r="C51" t="s">
         <v>18</v>
@@ -2808,7 +2839,7 @@
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="24"/>
+      <c r="A52" s="27"/>
       <c r="B52" s="19"/>
       <c r="C52" t="s">
         <v>19</v>
@@ -2818,7 +2849,7 @@
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="24"/>
+      <c r="A53" s="27"/>
       <c r="B53" s="20"/>
       <c r="C53" s="8" t="s">
         <v>20</v>
@@ -2828,7 +2859,7 @@
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" s="24"/>
+      <c r="A54" s="27"/>
       <c r="B54" s="18" t="s">
         <v>14</v>
       </c>
@@ -2840,7 +2871,7 @@
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" s="24"/>
+      <c r="A55" s="27"/>
       <c r="B55" s="19"/>
       <c r="C55" t="s">
         <v>18</v>
@@ -2850,7 +2881,7 @@
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" s="24"/>
+      <c r="A56" s="27"/>
       <c r="B56" s="19"/>
       <c r="C56" t="s">
         <v>19</v>
@@ -2860,7 +2891,7 @@
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" s="24"/>
+      <c r="A57" s="27"/>
       <c r="B57" s="20"/>
       <c r="C57" s="8" t="s">
         <v>20</v>
@@ -2870,7 +2901,7 @@
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A58" s="24"/>
+      <c r="A58" s="27"/>
       <c r="B58" s="18" t="s">
         <v>15</v>
       </c>
@@ -2882,7 +2913,7 @@
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A59" s="24"/>
+      <c r="A59" s="27"/>
       <c r="B59" s="19"/>
       <c r="C59" t="s">
         <v>18</v>
@@ -2892,7 +2923,7 @@
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" s="24"/>
+      <c r="A60" s="27"/>
       <c r="B60" s="19"/>
       <c r="C60" t="s">
         <v>19</v>
@@ -2902,7 +2933,7 @@
       </c>
     </row>
     <row r="61" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="25"/>
+      <c r="A61" s="28"/>
       <c r="B61" s="21"/>
       <c r="C61" s="5" t="s">
         <v>20</v>
@@ -2912,7 +2943,7 @@
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="26" t="s">
+      <c r="A62" s="22" t="s">
         <v>6</v>
       </c>
       <c r="B62" s="17" t="s">
@@ -2926,7 +2957,7 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="27"/>
+      <c r="A63" s="23"/>
       <c r="B63" s="12"/>
       <c r="C63" t="s">
         <v>18</v>
@@ -2936,7 +2967,7 @@
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="27"/>
+      <c r="A64" s="23"/>
       <c r="B64" s="12"/>
       <c r="C64" t="s">
         <v>19</v>
@@ -2946,7 +2977,7 @@
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A65" s="27"/>
+      <c r="A65" s="23"/>
       <c r="B65" s="13"/>
       <c r="C65" s="8" t="s">
         <v>20</v>
@@ -2956,7 +2987,7 @@
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" s="27"/>
+      <c r="A66" s="23"/>
       <c r="B66" s="11" t="s">
         <v>12</v>
       </c>
@@ -2968,7 +2999,7 @@
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" s="27"/>
+      <c r="A67" s="23"/>
       <c r="B67" s="12"/>
       <c r="C67" t="s">
         <v>18</v>
@@ -2978,7 +3009,7 @@
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="27"/>
+      <c r="A68" s="23"/>
       <c r="B68" s="12"/>
       <c r="C68" t="s">
         <v>19</v>
@@ -2988,7 +3019,7 @@
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" s="27"/>
+      <c r="A69" s="23"/>
       <c r="B69" s="13"/>
       <c r="C69" s="8" t="s">
         <v>20</v>
@@ -2998,7 +3029,7 @@
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="27"/>
+      <c r="A70" s="23"/>
       <c r="B70" s="11" t="s">
         <v>14</v>
       </c>
@@ -3010,7 +3041,7 @@
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" s="27"/>
+      <c r="A71" s="23"/>
       <c r="B71" s="12"/>
       <c r="C71" t="s">
         <v>18</v>
@@ -3020,7 +3051,7 @@
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A72" s="27"/>
+      <c r="A72" s="23"/>
       <c r="B72" s="12"/>
       <c r="C72" t="s">
         <v>19</v>
@@ -3030,7 +3061,7 @@
       </c>
     </row>
     <row r="73" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="28"/>
+      <c r="A73" s="24"/>
       <c r="B73" s="16"/>
       <c r="C73" s="5" t="s">
         <v>20</v>
@@ -3040,7 +3071,7 @@
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="26" t="s">
+      <c r="A74" s="22" t="s">
         <v>7</v>
       </c>
       <c r="B74" s="17" t="s">
@@ -3054,7 +3085,7 @@
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="27"/>
+      <c r="A75" s="23"/>
       <c r="B75" s="12"/>
       <c r="C75" t="s">
         <v>18</v>
@@ -3064,7 +3095,7 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="27"/>
+      <c r="A76" s="23"/>
       <c r="B76" s="12"/>
       <c r="C76" t="s">
         <v>19</v>
@@ -3074,7 +3105,7 @@
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="27"/>
+      <c r="A77" s="23"/>
       <c r="B77" s="13"/>
       <c r="C77" s="8" t="s">
         <v>20</v>
@@ -3084,7 +3115,7 @@
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="27"/>
+      <c r="A78" s="23"/>
       <c r="B78" s="11" t="s">
         <v>9</v>
       </c>
@@ -3096,7 +3127,7 @@
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A79" s="27"/>
+      <c r="A79" s="23"/>
       <c r="B79" s="12"/>
       <c r="C79" t="s">
         <v>18</v>
@@ -3106,7 +3137,7 @@
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" s="27"/>
+      <c r="A80" s="23"/>
       <c r="B80" s="12"/>
       <c r="C80" t="s">
         <v>19</v>
@@ -3116,7 +3147,7 @@
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A81" s="27"/>
+      <c r="A81" s="23"/>
       <c r="B81" s="13"/>
       <c r="C81" s="8" t="s">
         <v>20</v>
@@ -3126,7 +3157,7 @@
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" s="27"/>
+      <c r="A82" s="23"/>
       <c r="B82" s="11" t="s">
         <v>10</v>
       </c>
@@ -3138,7 +3169,7 @@
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" s="27"/>
+      <c r="A83" s="23"/>
       <c r="B83" s="12"/>
       <c r="C83" t="s">
         <v>18</v>
@@ -3148,7 +3179,7 @@
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" s="27"/>
+      <c r="A84" s="23"/>
       <c r="B84" s="12"/>
       <c r="C84" t="s">
         <v>19</v>
@@ -3158,7 +3189,7 @@
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A85" s="27"/>
+      <c r="A85" s="23"/>
       <c r="B85" s="13"/>
       <c r="C85" s="8" t="s">
         <v>20</v>
@@ -3168,7 +3199,7 @@
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A86" s="27"/>
+      <c r="A86" s="23"/>
       <c r="B86" s="11" t="s">
         <v>11</v>
       </c>
@@ -3180,7 +3211,7 @@
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A87" s="27"/>
+      <c r="A87" s="23"/>
       <c r="B87" s="12"/>
       <c r="C87" t="s">
         <v>18</v>
@@ -3190,7 +3221,7 @@
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A88" s="27"/>
+      <c r="A88" s="23"/>
       <c r="B88" s="12"/>
       <c r="C88" t="s">
         <v>19</v>
@@ -3200,7 +3231,7 @@
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A89" s="27"/>
+      <c r="A89" s="23"/>
       <c r="B89" s="13"/>
       <c r="C89" s="8" t="s">
         <v>20</v>
@@ -3210,7 +3241,7 @@
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A90" s="27"/>
+      <c r="A90" s="23"/>
       <c r="B90" s="11" t="s">
         <v>12</v>
       </c>
@@ -3222,7 +3253,7 @@
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A91" s="27"/>
+      <c r="A91" s="23"/>
       <c r="B91" s="12"/>
       <c r="C91" t="s">
         <v>18</v>
@@ -3232,7 +3263,7 @@
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A92" s="27"/>
+      <c r="A92" s="23"/>
       <c r="B92" s="12"/>
       <c r="C92" t="s">
         <v>19</v>
@@ -3242,7 +3273,7 @@
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A93" s="27"/>
+      <c r="A93" s="23"/>
       <c r="B93" s="13"/>
       <c r="C93" s="8" t="s">
         <v>20</v>
@@ -3252,7 +3283,7 @@
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A94" s="27"/>
+      <c r="A94" s="23"/>
       <c r="B94" s="11" t="s">
         <v>13</v>
       </c>
@@ -3264,7 +3295,7 @@
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A95" s="27"/>
+      <c r="A95" s="23"/>
       <c r="B95" s="12"/>
       <c r="C95" t="s">
         <v>18</v>
@@ -3274,7 +3305,7 @@
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A96" s="27"/>
+      <c r="A96" s="23"/>
       <c r="B96" s="12"/>
       <c r="C96" t="s">
         <v>19</v>
@@ -3284,7 +3315,7 @@
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A97" s="27"/>
+      <c r="A97" s="23"/>
       <c r="B97" s="13"/>
       <c r="C97" s="8" t="s">
         <v>20</v>
@@ -3294,7 +3325,7 @@
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A98" s="27"/>
+      <c r="A98" s="23"/>
       <c r="B98" s="11" t="s">
         <v>14</v>
       </c>
@@ -3306,7 +3337,7 @@
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A99" s="27"/>
+      <c r="A99" s="23"/>
       <c r="B99" s="12"/>
       <c r="C99" t="s">
         <v>18</v>
@@ -3316,7 +3347,7 @@
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A100" s="27"/>
+      <c r="A100" s="23"/>
       <c r="B100" s="12"/>
       <c r="C100" t="s">
         <v>19</v>
@@ -3326,7 +3357,7 @@
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A101" s="27"/>
+      <c r="A101" s="23"/>
       <c r="B101" s="13"/>
       <c r="C101" s="8" t="s">
         <v>20</v>
@@ -3336,7 +3367,7 @@
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A102" s="27"/>
+      <c r="A102" s="23"/>
       <c r="B102" s="11" t="s">
         <v>15</v>
       </c>
@@ -3348,7 +3379,7 @@
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A103" s="27"/>
+      <c r="A103" s="23"/>
       <c r="B103" s="12"/>
       <c r="C103" t="s">
         <v>18</v>
@@ -3358,7 +3389,7 @@
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A104" s="27"/>
+      <c r="A104" s="23"/>
       <c r="B104" s="12"/>
       <c r="C104" t="s">
         <v>19</v>
@@ -3368,7 +3399,7 @@
       </c>
     </row>
     <row r="105" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="28"/>
+      <c r="A105" s="24"/>
       <c r="B105" s="16"/>
       <c r="C105" s="5" t="s">
         <v>20</v>
@@ -3378,7 +3409,7 @@
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A106" s="26" t="s">
+      <c r="A106" s="22" t="s">
         <v>8</v>
       </c>
       <c r="B106" s="17" t="s">
@@ -3392,7 +3423,7 @@
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A107" s="27"/>
+      <c r="A107" s="23"/>
       <c r="B107" s="12"/>
       <c r="C107" t="s">
         <v>18</v>
@@ -3402,7 +3433,7 @@
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A108" s="27"/>
+      <c r="A108" s="23"/>
       <c r="B108" s="12"/>
       <c r="C108" t="s">
         <v>19</v>
@@ -3412,7 +3443,7 @@
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A109" s="27"/>
+      <c r="A109" s="23"/>
       <c r="B109" s="13"/>
       <c r="C109" s="8" t="s">
         <v>20</v>
@@ -3422,7 +3453,7 @@
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A110" s="27"/>
+      <c r="A110" s="23"/>
       <c r="B110" s="11" t="s">
         <v>9</v>
       </c>
@@ -3434,7 +3465,7 @@
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A111" s="27"/>
+      <c r="A111" s="23"/>
       <c r="B111" s="12"/>
       <c r="C111" t="s">
         <v>18</v>
@@ -3444,7 +3475,7 @@
       </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A112" s="27"/>
+      <c r="A112" s="23"/>
       <c r="B112" s="12"/>
       <c r="C112" t="s">
         <v>19</v>
@@ -3454,7 +3485,7 @@
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A113" s="27"/>
+      <c r="A113" s="23"/>
       <c r="B113" s="13"/>
       <c r="C113" s="8" t="s">
         <v>20</v>
@@ -3464,7 +3495,7 @@
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A114" s="27"/>
+      <c r="A114" s="23"/>
       <c r="B114" s="11" t="s">
         <v>10</v>
       </c>
@@ -3476,7 +3507,7 @@
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A115" s="27"/>
+      <c r="A115" s="23"/>
       <c r="B115" s="12"/>
       <c r="C115" t="s">
         <v>18</v>
@@ -3486,7 +3517,7 @@
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A116" s="27"/>
+      <c r="A116" s="23"/>
       <c r="B116" s="12"/>
       <c r="C116" t="s">
         <v>19</v>
@@ -3496,7 +3527,7 @@
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A117" s="27"/>
+      <c r="A117" s="23"/>
       <c r="B117" s="13"/>
       <c r="C117" s="8" t="s">
         <v>20</v>
@@ -3506,7 +3537,7 @@
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A118" s="27"/>
+      <c r="A118" s="23"/>
       <c r="B118" s="11" t="s">
         <v>11</v>
       </c>
@@ -3518,7 +3549,7 @@
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A119" s="27"/>
+      <c r="A119" s="23"/>
       <c r="B119" s="12"/>
       <c r="C119" t="s">
         <v>18</v>
@@ -3528,7 +3559,7 @@
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A120" s="27"/>
+      <c r="A120" s="23"/>
       <c r="B120" s="12"/>
       <c r="C120" t="s">
         <v>19</v>
@@ -3538,7 +3569,7 @@
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A121" s="27"/>
+      <c r="A121" s="23"/>
       <c r="B121" s="13"/>
       <c r="C121" s="8" t="s">
         <v>20</v>
@@ -3548,7 +3579,7 @@
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A122" s="27"/>
+      <c r="A122" s="23"/>
       <c r="B122" s="11" t="s">
         <v>12</v>
       </c>
@@ -3560,7 +3591,7 @@
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A123" s="27"/>
+      <c r="A123" s="23"/>
       <c r="B123" s="12"/>
       <c r="C123" t="s">
         <v>18</v>
@@ -3570,7 +3601,7 @@
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A124" s="27"/>
+      <c r="A124" s="23"/>
       <c r="B124" s="12"/>
       <c r="C124" t="s">
         <v>19</v>
@@ -3580,7 +3611,7 @@
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A125" s="27"/>
+      <c r="A125" s="23"/>
       <c r="B125" s="13"/>
       <c r="C125" s="8" t="s">
         <v>20</v>
@@ -3590,7 +3621,7 @@
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A126" s="27"/>
+      <c r="A126" s="23"/>
       <c r="B126" s="11" t="s">
         <v>13</v>
       </c>
@@ -3602,7 +3633,7 @@
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A127" s="27"/>
+      <c r="A127" s="23"/>
       <c r="B127" s="12"/>
       <c r="C127" t="s">
         <v>18</v>
@@ -3612,7 +3643,7 @@
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A128" s="27"/>
+      <c r="A128" s="23"/>
       <c r="B128" s="12"/>
       <c r="C128" t="s">
         <v>19</v>
@@ -3622,7 +3653,7 @@
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A129" s="27"/>
+      <c r="A129" s="23"/>
       <c r="B129" s="13"/>
       <c r="C129" s="8" t="s">
         <v>20</v>
@@ -3632,7 +3663,7 @@
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A130" s="27"/>
+      <c r="A130" s="23"/>
       <c r="B130" s="11" t="s">
         <v>14</v>
       </c>
@@ -3644,7 +3675,7 @@
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A131" s="27"/>
+      <c r="A131" s="23"/>
       <c r="B131" s="14"/>
       <c r="C131" t="s">
         <v>18</v>
@@ -3654,7 +3685,7 @@
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A132" s="27"/>
+      <c r="A132" s="23"/>
       <c r="B132" s="14"/>
       <c r="C132" t="s">
         <v>19</v>
@@ -3664,7 +3695,7 @@
       </c>
     </row>
     <row r="133" spans="1:4" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A133" s="28"/>
+      <c r="A133" s="24"/>
       <c r="B133" s="15"/>
       <c r="C133" s="5" t="s">
         <v>20</v>
@@ -3715,13 +3746,8 @@
     <mergeCell ref="B26:B29"/>
   </mergeCells>
   <conditionalFormatting sqref="D2:D133">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0.3"/>
-        <color theme="6" tint="0.39997558519241921"/>
-        <color theme="9" tint="0.39997558519241921"/>
-      </colorScale>
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
+      <formula>0.3</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>